<commit_message>
feat: LP register bot updated
</commit_message>
<xml_diff>
--- a/98 - Excels/Cadastro-LPs.xlsx
+++ b/98 - Excels/Cadastro-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\98 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4E3545-EB2E-422E-9431-4A46FE8A11F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AE8BF7-A840-4F82-BC41-232E62516C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Status</t>
   </si>
@@ -28,33 +28,12 @@
     <t>Data</t>
   </si>
   <si>
-    <t>4713400000</t>
-  </si>
-  <si>
-    <t>685531</t>
-  </si>
-  <si>
-    <t>LP-054431</t>
-  </si>
-  <si>
     <t>Objeto de Liquidação</t>
   </si>
   <si>
     <t>Part Number</t>
   </si>
   <si>
-    <t>Rodrigo Melo</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>Novo - Série 0196</t>
-  </si>
-  <si>
-    <t>QMM</t>
-  </si>
-  <si>
     <t>Prazo Final</t>
   </si>
   <si>
@@ -80,6 +59,18 @@
   </si>
   <si>
     <t>Nota PM</t>
+  </si>
+  <si>
+    <t>Yesica Gonzalez</t>
+  </si>
+  <si>
+    <t>bucha guia</t>
+  </si>
+  <si>
+    <t>DOUGLAS</t>
+  </si>
+  <si>
+    <t>LP-054888</t>
   </si>
 </sst>
 </file>
@@ -488,37 +479,37 @@
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="J1" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>0</v>
@@ -526,40 +517,40 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
-        <v>46027</v>
+        <v>46050</v>
       </c>
       <c r="B2" s="4">
-        <v>46125</v>
+        <v>46122</v>
       </c>
       <c r="C2" s="7">
-        <v>14178948</v>
+        <v>14193317</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>8</v>
+        <v>13</v>
+      </c>
+      <c r="E2" s="5">
+        <v>685541</v>
+      </c>
+      <c r="F2" s="5">
+        <v>19</v>
       </c>
       <c r="G2" s="5">
-        <v>1</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="H2" s="5">
+        <v>4729401967</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K2" s="5">
-        <v>2000</v>
+        <v>4400</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: LP-Register bot updated
</commit_message>
<xml_diff>
--- a/98 - Excels/Cadastro-LPs.xlsx
+++ b/98 - Excels/Cadastro-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\98 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C8A4C4-CDA5-4EAE-ADC5-687C642AD9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6BA4C43-ADEA-41BE-8DE9-33D1EBAAA7FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>Status</t>
   </si>
@@ -64,13 +64,37 @@
     <t>Yesica Gonzalez</t>
   </si>
   <si>
-    <t>bucha guia</t>
-  </si>
-  <si>
-    <t>DOUGLAS</t>
-  </si>
-  <si>
-    <t>LP-054888</t>
+    <t>05.01.2026</t>
+  </si>
+  <si>
+    <t>20.03.2026</t>
+  </si>
+  <si>
+    <t>IP 685487 Pino d suporte Ret.Fortuna ⌀10</t>
+  </si>
+  <si>
+    <t>DONI- 2803</t>
+  </si>
+  <si>
+    <t>1 200,00</t>
+  </si>
+  <si>
+    <t>LP-054499</t>
+  </si>
+  <si>
+    <t>07.01.2026</t>
+  </si>
+  <si>
+    <t>1+/11,48 -0,006</t>
+  </si>
+  <si>
+    <t>VIM6CT</t>
+  </si>
+  <si>
+    <t>2 400,00</t>
+  </si>
+  <si>
+    <t>LP-054692</t>
   </si>
 </sst>
 </file>
@@ -457,18 +481,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="38" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6.42578125" bestFit="1" customWidth="1"/>
@@ -516,41 +541,79 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>46050</v>
-      </c>
-      <c r="B2" s="4">
-        <v>46122</v>
+      <c r="A2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="C2" s="7">
-        <v>14193317</v>
+        <v>14178673</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E2" s="5">
-        <v>685541</v>
+        <v>685487</v>
       </c>
       <c r="F2" s="5">
         <v>19</v>
       </c>
       <c r="G2" s="5">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H2" s="5">
-        <v>4729401967</v>
+        <v>4710200220</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="5">
-        <v>4400</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>16</v>
+      <c r="C3" s="7">
+        <v>14180350</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5">
+        <v>685401</v>
+      </c>
+      <c r="F3" s="5">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5">
+        <v>4711401345</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: lp register updated and testing
</commit_message>
<xml_diff>
--- a/98 - Excels/Cadastro-LPs.xlsx
+++ b/98 - Excels/Cadastro-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feb3ct\Desktop\PyAutomateSAP\98 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A3FA9B-AC25-4989-8315-407E784FD4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8815FF70-AF72-41BC-9A0F-A03E1030CF00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -595,15 +595,6 @@
     <t>Status CN21</t>
   </si>
   <si>
-    <t>LP055085</t>
-  </si>
-  <si>
-    <t>LP055087</t>
-  </si>
-  <si>
-    <t>LP055097</t>
-  </si>
-  <si>
     <t>CAPA DE EXPULSOR</t>
   </si>
   <si>
@@ -616,147 +607,27 @@
     <t>6 060,00</t>
   </si>
   <si>
-    <t>LP055859</t>
-  </si>
-  <si>
-    <t>LP055086</t>
-  </si>
-  <si>
-    <t>LP055047</t>
-  </si>
-  <si>
-    <t>LP055092</t>
-  </si>
-  <si>
-    <t>LP055091</t>
-  </si>
-  <si>
-    <t>LP055089</t>
-  </si>
-  <si>
-    <t>LP055090</t>
-  </si>
-  <si>
-    <t>LP055088</t>
-  </si>
-  <si>
-    <t>LP055193</t>
-  </si>
-  <si>
-    <t>LP055061</t>
-  </si>
-  <si>
-    <t>LP055160</t>
-  </si>
-  <si>
-    <t>LP055239</t>
-  </si>
-  <si>
-    <t>LP055206</t>
-  </si>
-  <si>
-    <t>LP055204</t>
-  </si>
-  <si>
-    <t>LP055163</t>
-  </si>
-  <si>
-    <t>LP055156</t>
-  </si>
-  <si>
-    <t>LP055158</t>
-  </si>
-  <si>
-    <t>LP055164</t>
-  </si>
-  <si>
-    <t>LP055100</t>
-  </si>
-  <si>
-    <t>LP055060</t>
-  </si>
-  <si>
-    <t>LP055095</t>
-  </si>
-  <si>
-    <t>LP055208</t>
-  </si>
-  <si>
-    <t>LP055162</t>
-  </si>
-  <si>
-    <t>LP055161</t>
-  </si>
-  <si>
-    <t>LP055155</t>
-  </si>
-  <si>
-    <t>LP055099</t>
-  </si>
-  <si>
-    <t>LP055154</t>
-  </si>
-  <si>
     <t>CtP/MFE31</t>
   </si>
   <si>
-    <t>LP055411</t>
-  </si>
-  <si>
-    <t>LP055237</t>
-  </si>
-  <si>
-    <t>LP055614</t>
-  </si>
-  <si>
-    <t>LP055616</t>
-  </si>
-  <si>
-    <t>LP055393</t>
-  </si>
-  <si>
     <t>Dispositivo bloco de pressão</t>
   </si>
   <si>
-    <t>LP055613</t>
-  </si>
-  <si>
     <t>CtP/MFW11-B</t>
   </si>
   <si>
-    <t>LP055461</t>
-  </si>
-  <si>
-    <t>LP055437</t>
-  </si>
-  <si>
-    <t>LP055392</t>
-  </si>
-  <si>
-    <t>LP055612</t>
-  </si>
-  <si>
-    <t>LP055609</t>
-  </si>
-  <si>
     <t>Ponteira Blaichach</t>
   </si>
   <si>
     <t>1 050,00</t>
   </si>
   <si>
-    <t>LP055611</t>
-  </si>
-  <si>
     <t>Posição 4</t>
   </si>
   <si>
     <t>1 920,00</t>
   </si>
   <si>
-    <t>LP055610</t>
-  </si>
-  <si>
     <t>4781700221/31</t>
   </si>
   <si>
@@ -766,36 +637,12 @@
     <t>9 200,00</t>
   </si>
   <si>
-    <t>LP055637</t>
-  </si>
-  <si>
     <t>Disp. Robodril</t>
   </si>
   <si>
     <t>11 700,00</t>
   </si>
   <si>
-    <t>LP055631</t>
-  </si>
-  <si>
-    <t>LP055420</t>
-  </si>
-  <si>
-    <t>LP055415</t>
-  </si>
-  <si>
-    <t>LP055419</t>
-  </si>
-  <si>
-    <t>LP055416</t>
-  </si>
-  <si>
-    <t>LP055417</t>
-  </si>
-  <si>
-    <t>LP055418</t>
-  </si>
-  <si>
     <t>Pino UVA</t>
   </si>
   <si>
@@ -805,126 +652,42 @@
     <t>2 800,00</t>
   </si>
   <si>
-    <t>LP055898</t>
-  </si>
-  <si>
-    <t>LP055899</t>
-  </si>
-  <si>
-    <t>LP055430</t>
-  </si>
-  <si>
-    <t>LP055424</t>
-  </si>
-  <si>
-    <t>LP055434</t>
-  </si>
-  <si>
-    <t>LP055394</t>
-  </si>
-  <si>
-    <t>LP055432</t>
-  </si>
-  <si>
-    <t>LP055431</t>
-  </si>
-  <si>
-    <t>LP055428</t>
-  </si>
-  <si>
-    <t>LP055433</t>
-  </si>
-  <si>
-    <t>LP055429</t>
-  </si>
-  <si>
-    <t>LP055395</t>
-  </si>
-  <si>
-    <t>LP055396</t>
-  </si>
-  <si>
-    <t>LP055427</t>
-  </si>
-  <si>
     <t>DU 685421 Conexão de usinagem HE</t>
   </si>
   <si>
-    <t>LP055522</t>
-  </si>
-  <si>
-    <t>LP055462</t>
-  </si>
-  <si>
-    <t>LP055463</t>
-  </si>
-  <si>
-    <t>LP055436</t>
-  </si>
-  <si>
-    <t>LP055464</t>
-  </si>
-  <si>
     <t>DU 685434 Chapa d alimentação acabamen.</t>
   </si>
   <si>
     <t>1 320,00</t>
   </si>
   <si>
-    <t>LP055523</t>
-  </si>
-  <si>
     <t>DU 685434 Bico de refrigeração POSIÇÃO 1</t>
   </si>
   <si>
     <t>3 280,00</t>
   </si>
   <si>
-    <t>LP055524</t>
-  </si>
-  <si>
     <t>CtP/TEF1</t>
   </si>
   <si>
-    <t>LP055457</t>
-  </si>
-  <si>
     <t>encosto da thielenhaus</t>
   </si>
   <si>
-    <t>LP055934</t>
-  </si>
-  <si>
-    <t>LP055460</t>
-  </si>
-  <si>
-    <t>LP055450</t>
-  </si>
-  <si>
     <t>DU 685411 POS 1 Sistema d Alimen.Supfina</t>
   </si>
   <si>
     <t>3 560,00</t>
   </si>
   <si>
-    <t>LP055595</t>
-  </si>
-  <si>
     <t>DU 685411 POS 3 Sistema d Alimen.Supfina</t>
   </si>
   <si>
-    <t>LP055596</t>
-  </si>
-  <si>
     <t>DU 685411 POS23 Sistema d Alimen.Supfina</t>
   </si>
   <si>
     <t>10 360,00</t>
   </si>
   <si>
-    <t>LP055597</t>
-  </si>
-  <si>
     <t>23.02.2026</t>
   </si>
   <si>
@@ -934,48 +697,30 @@
     <t>Mandril rebolo Supfina - Fabricação</t>
   </si>
   <si>
-    <t>LP055636</t>
-  </si>
-  <si>
     <t>24.02.2026</t>
   </si>
   <si>
     <t>IP 685491 POSIÇÃO 8 bancada escovação.</t>
   </si>
   <si>
-    <t>LP055507</t>
-  </si>
-  <si>
     <t>DU 685412 POSIÇÃO 1 do pino Guiringuelli</t>
   </si>
   <si>
     <t>3 840,00</t>
   </si>
   <si>
-    <t>LP055519</t>
-  </si>
-  <si>
-    <t>LP007619-04-22</t>
-  </si>
-  <si>
     <t>Retrabalho da altura do magazine agulha</t>
   </si>
   <si>
     <t>JOSIANE OLIV</t>
   </si>
   <si>
-    <t>LP055513</t>
-  </si>
-  <si>
     <t>4729108882 POS1</t>
   </si>
   <si>
     <t>DU 685421 POSIÇÃO 1  do cabeçote AGIE</t>
   </si>
   <si>
-    <t>LP055517</t>
-  </si>
-  <si>
     <t>4729108882 POS7</t>
   </si>
   <si>
@@ -985,15 +730,9 @@
     <t>1 150,00</t>
   </si>
   <si>
-    <t>LP055518</t>
-  </si>
-  <si>
     <t>DU 685421 Conector ∅4/6</t>
   </si>
   <si>
-    <t>LP055521</t>
-  </si>
-  <si>
     <t>25.02.2026</t>
   </si>
   <si>
@@ -1003,45 +742,24 @@
     <t>DU 685421 Pino fixação bico S-POSIÇÃO 2</t>
   </si>
   <si>
-    <t>LP055536</t>
-  </si>
-  <si>
     <t>IP 685481 Castanha studer Válvula</t>
   </si>
   <si>
-    <t>LP055540</t>
-  </si>
-  <si>
     <t>Castanha da placa</t>
   </si>
   <si>
     <t>4 560,00</t>
   </si>
   <si>
-    <t>LP055556</t>
-  </si>
-  <si>
     <t>GARRA POSIÇÃO 13</t>
   </si>
   <si>
     <t>2 440,00</t>
   </si>
   <si>
-    <t>LP055554</t>
-  </si>
-  <si>
     <t>Dispositivo DHK</t>
   </si>
   <si>
-    <t>LP055553</t>
-  </si>
-  <si>
-    <t>LP055555</t>
-  </si>
-  <si>
-    <t>LP055552</t>
-  </si>
-  <si>
     <t>4710900878 P01 F2</t>
   </si>
   <si>
@@ -1054,63 +772,24 @@
     <t>CtP/MFW13-A</t>
   </si>
   <si>
-    <t>LP055537</t>
-  </si>
-  <si>
-    <t>LP055546</t>
-  </si>
-  <si>
-    <t>LP055551</t>
-  </si>
-  <si>
-    <t>LP055550</t>
-  </si>
-  <si>
     <t>Cone da montagem</t>
   </si>
   <si>
-    <t>LP055549</t>
-  </si>
-  <si>
     <t>DU 685411 Pinça d Alimentação Haste Chei</t>
   </si>
   <si>
     <t>2 720,00</t>
   </si>
   <si>
-    <t>LP055526</t>
-  </si>
-  <si>
     <t>IP 685484 Rebolo borazon Pistão A/P</t>
   </si>
   <si>
-    <t>LP055541</t>
-  </si>
-  <si>
-    <t>LP055542</t>
-  </si>
-  <si>
-    <t>LP055544</t>
-  </si>
-  <si>
-    <t>LP055545</t>
-  </si>
-  <si>
-    <t>LP055547</t>
-  </si>
-  <si>
-    <t>LP055548</t>
-  </si>
-  <si>
     <t>4728700097 POS 5</t>
   </si>
   <si>
     <t>IP 685484 Prisma de apoio pistão P</t>
   </si>
   <si>
-    <t>LP055543</t>
-  </si>
-  <si>
     <t>26.02.2026</t>
   </si>
   <si>
@@ -1120,15 +799,9 @@
     <t>1 500,00</t>
   </si>
   <si>
-    <t>LP055534</t>
-  </si>
-  <si>
     <t>DU 685421 Guia de eletrodo AGIEs</t>
   </si>
   <si>
-    <t>LP055535</t>
-  </si>
-  <si>
     <t>Base completa - Todas posições</t>
   </si>
   <si>
@@ -1141,27 +814,15 @@
     <t>8 300,00</t>
   </si>
   <si>
-    <t>LP055575</t>
-  </si>
-  <si>
     <t>9 960,00</t>
   </si>
   <si>
-    <t>LP055576</t>
-  </si>
-  <si>
     <t>DU 685411 Garra de alimentação HTT 3362</t>
   </si>
   <si>
-    <t>LP055530</t>
-  </si>
-  <si>
     <t>DU 685411 Garra de alimentação HTT 3352</t>
   </si>
   <si>
-    <t>LP055531</t>
-  </si>
-  <si>
     <t>4729107609 POS 9</t>
   </si>
   <si>
@@ -1171,18 +832,12 @@
     <t>1 780,00</t>
   </si>
   <si>
-    <t>LP055629</t>
-  </si>
-  <si>
     <t>4729107609 POS 12</t>
   </si>
   <si>
     <t>IP 685485 POSIÇÃO 12 Sistema de aliment.</t>
   </si>
   <si>
-    <t>LP055630</t>
-  </si>
-  <si>
     <t>27.02.2026</t>
   </si>
   <si>
@@ -1192,108 +847,54 @@
     <t>IP 685010 Borracha de vedação ATEQ POS11</t>
   </si>
   <si>
-    <t>LP055625</t>
-  </si>
-  <si>
     <t>IP 685482 Eletrodo ecm corpo CRIN/LE</t>
   </si>
   <si>
-    <t>LP055626</t>
-  </si>
-  <si>
     <t>IP 685482 Eletrodo POS 1 ecm corpo CRIN</t>
   </si>
   <si>
-    <t>LP055627</t>
-  </si>
-  <si>
     <t>DU 685434 Garra supfina Turquia acabamen</t>
   </si>
   <si>
     <t>4 080,00</t>
   </si>
   <si>
-    <t>LP055570</t>
-  </si>
-  <si>
     <t>Parafuso Robodril posição 03</t>
   </si>
   <si>
-    <t>LP055622</t>
-  </si>
-  <si>
     <t>Suporte do alimentador</t>
   </si>
   <si>
     <t>3 690,00</t>
   </si>
   <si>
-    <t>LP055638</t>
-  </si>
-  <si>
     <t>DU 685434 Pino Centralizador Lavador.Glu</t>
   </si>
   <si>
-    <t>LP055571</t>
-  </si>
-  <si>
     <t>DU 685434 Pino posicionador lavadora Glu</t>
   </si>
   <si>
     <t>3 200,00</t>
   </si>
   <si>
-    <t>LP055572</t>
-  </si>
-  <si>
     <t>DU 685433 Arruela bancada de montag Bico</t>
   </si>
   <si>
-    <t>LP055569</t>
-  </si>
-  <si>
     <t>Porta bucha</t>
   </si>
   <si>
-    <t>LP055620</t>
-  </si>
-  <si>
     <t>DU 685411 Pino de aliment. Nomyline 4mm</t>
   </si>
   <si>
-    <t>LP055581</t>
-  </si>
-  <si>
-    <t>LP055619</t>
-  </si>
-  <si>
-    <t>LP055621</t>
-  </si>
-  <si>
     <t>IP 685072 Pinça CIL P7/P8/R/TICs  ⌀12</t>
   </si>
   <si>
-    <t>LP055623</t>
-  </si>
-  <si>
     <t>IP 685485 Arrastador de pallet Brunidora</t>
   </si>
   <si>
-    <t>LP055624</t>
-  </si>
-  <si>
     <t>IP 685485 Vareta de presença Brunidoras.</t>
   </si>
   <si>
-    <t>LP055580</t>
-  </si>
-  <si>
-    <t>LP055618</t>
-  </si>
-  <si>
-    <t>LP055617</t>
-  </si>
-  <si>
     <t>ANEXO</t>
   </si>
   <si>
@@ -1303,9 +904,6 @@
     <t>DONI/VELLUD</t>
   </si>
   <si>
-    <t>LP055589</t>
-  </si>
-  <si>
     <t>28.02.2026</t>
   </si>
   <si>
@@ -1315,39 +913,21 @@
     <t>1 600,00</t>
   </si>
   <si>
-    <t>LP055600</t>
-  </si>
-  <si>
-    <t>LP055628</t>
-  </si>
-  <si>
     <t>12 850,00</t>
   </si>
   <si>
-    <t>LP055687</t>
-  </si>
-  <si>
     <t>Dispositivo posição 01</t>
   </si>
   <si>
     <t>3 720,00</t>
   </si>
   <si>
-    <t>LP055742</t>
-  </si>
-  <si>
     <t>TAGS POSIÇÃO 02</t>
   </si>
   <si>
-    <t>LP055598</t>
-  </si>
-  <si>
     <t>TAGS POSIÇÃO 01</t>
   </si>
   <si>
-    <t>LP055599</t>
-  </si>
-  <si>
     <t>02.03.2026</t>
   </si>
   <si>
@@ -1631,6 +1211,426 @@
   </si>
   <si>
     <t>LP-055910</t>
+  </si>
+  <si>
+    <t>LP-055085</t>
+  </si>
+  <si>
+    <t>LP-055087</t>
+  </si>
+  <si>
+    <t>LP-055097</t>
+  </si>
+  <si>
+    <t>LP-055859</t>
+  </si>
+  <si>
+    <t>LP-055086</t>
+  </si>
+  <si>
+    <t>LP-055047</t>
+  </si>
+  <si>
+    <t>LP-055092</t>
+  </si>
+  <si>
+    <t>LP-055091</t>
+  </si>
+  <si>
+    <t>LP-055089</t>
+  </si>
+  <si>
+    <t>LP-055090</t>
+  </si>
+  <si>
+    <t>LP-055088</t>
+  </si>
+  <si>
+    <t>LP-055193</t>
+  </si>
+  <si>
+    <t>LP-055061</t>
+  </si>
+  <si>
+    <t>LP-055160</t>
+  </si>
+  <si>
+    <t>LP-055239</t>
+  </si>
+  <si>
+    <t>LP-055206</t>
+  </si>
+  <si>
+    <t>LP-055204</t>
+  </si>
+  <si>
+    <t>LP-055163</t>
+  </si>
+  <si>
+    <t>LP-055156</t>
+  </si>
+  <si>
+    <t>LP-055158</t>
+  </si>
+  <si>
+    <t>LP-055164</t>
+  </si>
+  <si>
+    <t>LP-055100</t>
+  </si>
+  <si>
+    <t>LP-055060</t>
+  </si>
+  <si>
+    <t>LP-055095</t>
+  </si>
+  <si>
+    <t>LP-055208</t>
+  </si>
+  <si>
+    <t>LP-055162</t>
+  </si>
+  <si>
+    <t>LP-055161</t>
+  </si>
+  <si>
+    <t>LP-055155</t>
+  </si>
+  <si>
+    <t>LP-055099</t>
+  </si>
+  <si>
+    <t>LP-055154</t>
+  </si>
+  <si>
+    <t>LP-055411</t>
+  </si>
+  <si>
+    <t>LP-055237</t>
+  </si>
+  <si>
+    <t>LP-055614</t>
+  </si>
+  <si>
+    <t>LP-055616</t>
+  </si>
+  <si>
+    <t>LP-055393</t>
+  </si>
+  <si>
+    <t>LP-055613</t>
+  </si>
+  <si>
+    <t>LP-055461</t>
+  </si>
+  <si>
+    <t>LP-055437</t>
+  </si>
+  <si>
+    <t>LP-055392</t>
+  </si>
+  <si>
+    <t>LP-055612</t>
+  </si>
+  <si>
+    <t>LP-055609</t>
+  </si>
+  <si>
+    <t>LP-055611</t>
+  </si>
+  <si>
+    <t>LP-055610</t>
+  </si>
+  <si>
+    <t>LP-055637</t>
+  </si>
+  <si>
+    <t>LP-055631</t>
+  </si>
+  <si>
+    <t>LP-055420</t>
+  </si>
+  <si>
+    <t>LP-055415</t>
+  </si>
+  <si>
+    <t>LP-055419</t>
+  </si>
+  <si>
+    <t>LP-055416</t>
+  </si>
+  <si>
+    <t>LP-055417</t>
+  </si>
+  <si>
+    <t>LP-055418</t>
+  </si>
+  <si>
+    <t>LP-055898</t>
+  </si>
+  <si>
+    <t>LP-055899</t>
+  </si>
+  <si>
+    <t>LP-055430</t>
+  </si>
+  <si>
+    <t>LP-055424</t>
+  </si>
+  <si>
+    <t>LP-055434</t>
+  </si>
+  <si>
+    <t>LP-055394</t>
+  </si>
+  <si>
+    <t>LP-055432</t>
+  </si>
+  <si>
+    <t>LP-055431</t>
+  </si>
+  <si>
+    <t>LP-055428</t>
+  </si>
+  <si>
+    <t>LP-055433</t>
+  </si>
+  <si>
+    <t>LP-055429</t>
+  </si>
+  <si>
+    <t>LP-055395</t>
+  </si>
+  <si>
+    <t>LP-055396</t>
+  </si>
+  <si>
+    <t>LP-055427</t>
+  </si>
+  <si>
+    <t>LP-055522</t>
+  </si>
+  <si>
+    <t>LP-055462</t>
+  </si>
+  <si>
+    <t>LP-055463</t>
+  </si>
+  <si>
+    <t>LP-055436</t>
+  </si>
+  <si>
+    <t>LP-055464</t>
+  </si>
+  <si>
+    <t>LP-055523</t>
+  </si>
+  <si>
+    <t>LP-055524</t>
+  </si>
+  <si>
+    <t>LP-055457</t>
+  </si>
+  <si>
+    <t>LP-055934</t>
+  </si>
+  <si>
+    <t>LP-055460</t>
+  </si>
+  <si>
+    <t>LP-055450</t>
+  </si>
+  <si>
+    <t>LP-055595</t>
+  </si>
+  <si>
+    <t>LP-055596</t>
+  </si>
+  <si>
+    <t>LP-055597</t>
+  </si>
+  <si>
+    <t>LP-055636</t>
+  </si>
+  <si>
+    <t>LP-055507</t>
+  </si>
+  <si>
+    <t>LP-055519</t>
+  </si>
+  <si>
+    <t>LP-007619-04-22</t>
+  </si>
+  <si>
+    <t>LP-055513</t>
+  </si>
+  <si>
+    <t>LP-055517</t>
+  </si>
+  <si>
+    <t>LP-055518</t>
+  </si>
+  <si>
+    <t>LP-055521</t>
+  </si>
+  <si>
+    <t>LP-055536</t>
+  </si>
+  <si>
+    <t>LP-055540</t>
+  </si>
+  <si>
+    <t>LP-055556</t>
+  </si>
+  <si>
+    <t>LP-055554</t>
+  </si>
+  <si>
+    <t>LP-055553</t>
+  </si>
+  <si>
+    <t>LP-055555</t>
+  </si>
+  <si>
+    <t>LP-055552</t>
+  </si>
+  <si>
+    <t>LP-055537</t>
+  </si>
+  <si>
+    <t>LP-055546</t>
+  </si>
+  <si>
+    <t>LP-055551</t>
+  </si>
+  <si>
+    <t>LP-055550</t>
+  </si>
+  <si>
+    <t>LP-055549</t>
+  </si>
+  <si>
+    <t>LP-055526</t>
+  </si>
+  <si>
+    <t>LP-055541</t>
+  </si>
+  <si>
+    <t>LP-055542</t>
+  </si>
+  <si>
+    <t>LP-055544</t>
+  </si>
+  <si>
+    <t>LP-055545</t>
+  </si>
+  <si>
+    <t>LP-055547</t>
+  </si>
+  <si>
+    <t>LP-055548</t>
+  </si>
+  <si>
+    <t>LP-055543</t>
+  </si>
+  <si>
+    <t>LP-055534</t>
+  </si>
+  <si>
+    <t>LP-055535</t>
+  </si>
+  <si>
+    <t>LP-055575</t>
+  </si>
+  <si>
+    <t>LP-055576</t>
+  </si>
+  <si>
+    <t>LP-055530</t>
+  </si>
+  <si>
+    <t>LP-055531</t>
+  </si>
+  <si>
+    <t>LP-055629</t>
+  </si>
+  <si>
+    <t>LP-055630</t>
+  </si>
+  <si>
+    <t>LP-055625</t>
+  </si>
+  <si>
+    <t>LP-055626</t>
+  </si>
+  <si>
+    <t>LP-055627</t>
+  </si>
+  <si>
+    <t>LP-055570</t>
+  </si>
+  <si>
+    <t>LP-055622</t>
+  </si>
+  <si>
+    <t>LP-055638</t>
+  </si>
+  <si>
+    <t>LP-055571</t>
+  </si>
+  <si>
+    <t>LP-055572</t>
+  </si>
+  <si>
+    <t>LP-055569</t>
+  </si>
+  <si>
+    <t>LP-055620</t>
+  </si>
+  <si>
+    <t>LP-055581</t>
+  </si>
+  <si>
+    <t>LP-055619</t>
+  </si>
+  <si>
+    <t>LP-055621</t>
+  </si>
+  <si>
+    <t>LP-055623</t>
+  </si>
+  <si>
+    <t>LP-055624</t>
+  </si>
+  <si>
+    <t>LP-055580</t>
+  </si>
+  <si>
+    <t>LP-055618</t>
+  </si>
+  <si>
+    <t>LP-055617</t>
+  </si>
+  <si>
+    <t>LP-055589</t>
+  </si>
+  <si>
+    <t>LP-055600</t>
+  </si>
+  <si>
+    <t>LP-055628</t>
+  </si>
+  <si>
+    <t>LP-055687</t>
+  </si>
+  <si>
+    <t>LP-055742</t>
+  </si>
+  <si>
+    <t>LP-055598</t>
+  </si>
+  <si>
+    <t>LP-055599</t>
   </si>
 </sst>
 </file>
@@ -3025,7 +3025,7 @@
         <v>82</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>191</v>
+        <v>397</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
@@ -3066,7 +3066,7 @@
         <v>84</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>192</v>
+        <v>398</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -3107,7 +3107,7 @@
         <v>86</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>193</v>
+        <v>399</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
@@ -3136,19 +3136,19 @@
         <v>4712001238</v>
       </c>
       <c r="I26" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="L26" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="J26" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="L26" s="5" t="s">
-        <v>197</v>
-      </c>
       <c r="M26" s="5" t="s">
-        <v>198</v>
+        <v>400</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
@@ -3189,7 +3189,7 @@
         <v>88</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>199</v>
+        <v>401</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
@@ -3230,7 +3230,7 @@
         <v>91</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>200</v>
+        <v>402</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
@@ -3271,7 +3271,7 @@
         <v>93</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>201</v>
+        <v>403</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
@@ -3312,7 +3312,7 @@
         <v>33</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>202</v>
+        <v>404</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
@@ -3353,7 +3353,7 @@
         <v>96</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>203</v>
+        <v>405</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -3394,7 +3394,7 @@
         <v>98</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>204</v>
+        <v>406</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
@@ -3435,7 +3435,7 @@
         <v>100</v>
       </c>
       <c r="M33" s="5" t="s">
-        <v>205</v>
+        <v>407</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
@@ -3476,7 +3476,7 @@
         <v>103</v>
       </c>
       <c r="M34" s="5" t="s">
-        <v>206</v>
+        <v>408</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
@@ -3517,7 +3517,7 @@
         <v>105</v>
       </c>
       <c r="M35" s="5" t="s">
-        <v>207</v>
+        <v>409</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
@@ -3558,7 +3558,7 @@
         <v>600</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>208</v>
+        <v>410</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
@@ -3599,7 +3599,7 @@
         <v>108</v>
       </c>
       <c r="M37" s="5" t="s">
-        <v>209</v>
+        <v>411</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
@@ -3640,7 +3640,7 @@
         <v>110</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>210</v>
+        <v>412</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
@@ -3681,7 +3681,7 @@
         <v>112</v>
       </c>
       <c r="M39" s="5" t="s">
-        <v>211</v>
+        <v>413</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
@@ -3722,7 +3722,7 @@
         <v>114</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>212</v>
+        <v>414</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
@@ -3763,7 +3763,7 @@
         <v>112</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>213</v>
+        <v>415</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
@@ -3804,7 +3804,7 @@
         <v>41</v>
       </c>
       <c r="M42" s="5" t="s">
-        <v>214</v>
+        <v>416</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
@@ -3845,7 +3845,7 @@
         <v>103</v>
       </c>
       <c r="M43" s="5" t="s">
-        <v>215</v>
+        <v>417</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
@@ -3886,7 +3886,7 @@
         <v>68</v>
       </c>
       <c r="M44" s="5" t="s">
-        <v>216</v>
+        <v>418</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
@@ -3927,7 +3927,7 @@
         <v>112</v>
       </c>
       <c r="M45" s="5" t="s">
-        <v>217</v>
+        <v>419</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
@@ -3968,7 +3968,7 @@
         <v>103</v>
       </c>
       <c r="M46" s="5" t="s">
-        <v>218</v>
+        <v>420</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
@@ -4009,7 +4009,7 @@
         <v>660</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>219</v>
+        <v>421</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
@@ -4050,7 +4050,7 @@
         <v>400</v>
       </c>
       <c r="M48" s="5" t="s">
-        <v>220</v>
+        <v>422</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>300</v>
       </c>
       <c r="M49" s="5" t="s">
-        <v>221</v>
+        <v>423</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
@@ -4132,7 +4132,7 @@
         <v>124</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>222</v>
+        <v>424</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
@@ -4173,7 +4173,7 @@
         <v>126</v>
       </c>
       <c r="M51" s="5" t="s">
-        <v>223</v>
+        <v>425</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
@@ -4214,7 +4214,7 @@
         <v>600</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>224</v>
+        <v>426</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
@@ -4249,13 +4249,13 @@
         <v>129</v>
       </c>
       <c r="K53" s="5" t="s">
-        <v>225</v>
+        <v>195</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>82</v>
       </c>
       <c r="M53" s="5" t="s">
-        <v>226</v>
+        <v>427</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
@@ -4296,7 +4296,7 @@
         <v>134</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>227</v>
+        <v>428</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
@@ -4337,7 +4337,7 @@
         <v>600</v>
       </c>
       <c r="M55" s="5" t="s">
-        <v>228</v>
+        <v>429</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
@@ -4378,7 +4378,7 @@
         <v>600</v>
       </c>
       <c r="M56" s="5" t="s">
-        <v>229</v>
+        <v>430</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
@@ -4419,7 +4419,7 @@
         <v>137</v>
       </c>
       <c r="M57" s="5" t="s">
-        <v>230</v>
+        <v>431</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
@@ -4448,7 +4448,7 @@
         <v>4723000024</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>231</v>
+        <v>196</v>
       </c>
       <c r="J58" s="5" t="s">
         <v>58</v>
@@ -4460,7 +4460,7 @@
         <v>33</v>
       </c>
       <c r="M58" s="5" t="s">
-        <v>232</v>
+        <v>432</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.25">
@@ -4495,13 +4495,13 @@
         <v>140</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="L59" s="5" t="s">
         <v>16</v>
       </c>
       <c r="M59" s="5" t="s">
-        <v>234</v>
+        <v>433</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.25">
@@ -4542,7 +4542,7 @@
         <v>143</v>
       </c>
       <c r="M60" s="5" t="s">
-        <v>235</v>
+        <v>434</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
@@ -4581,7 +4581,7 @@
         <v>330</v>
       </c>
       <c r="M61" s="5" t="s">
-        <v>236</v>
+        <v>435</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
@@ -4622,7 +4622,7 @@
         <v>600</v>
       </c>
       <c r="M62" s="5" t="s">
-        <v>237</v>
+        <v>436</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
@@ -4663,7 +4663,7 @@
         <v>600</v>
       </c>
       <c r="M63" s="5" t="s">
-        <v>238</v>
+        <v>437</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.25">
@@ -4692,7 +4692,7 @@
         <v>4729107684</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
       <c r="J64" s="5" t="s">
         <v>58</v>
@@ -4701,10 +4701,10 @@
         <v>185</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>240</v>
+        <v>199</v>
       </c>
       <c r="M64" s="5" t="s">
-        <v>241</v>
+        <v>438</v>
       </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
@@ -4733,7 +4733,7 @@
         <v>4728800293</v>
       </c>
       <c r="I65" s="5" t="s">
-        <v>242</v>
+        <v>200</v>
       </c>
       <c r="J65" s="5" t="s">
         <v>58</v>
@@ -4742,10 +4742,10 @@
         <v>185</v>
       </c>
       <c r="L65" s="5" t="s">
-        <v>243</v>
+        <v>201</v>
       </c>
       <c r="M65" s="5" t="s">
-        <v>244</v>
+        <v>439</v>
       </c>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.25">
@@ -4771,10 +4771,10 @@
         <v>10</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>245</v>
+        <v>202</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>246</v>
+        <v>203</v>
       </c>
       <c r="J66" s="5" t="s">
         <v>58</v>
@@ -4783,10 +4783,10 @@
         <v>185</v>
       </c>
       <c r="L66" s="5" t="s">
-        <v>247</v>
+        <v>204</v>
       </c>
       <c r="M66" s="5" t="s">
-        <v>248</v>
+        <v>440</v>
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
@@ -4815,7 +4815,7 @@
         <v>4727501921</v>
       </c>
       <c r="I67" s="5" t="s">
-        <v>249</v>
+        <v>205</v>
       </c>
       <c r="J67" s="5" t="s">
         <v>58</v>
@@ -4824,10 +4824,10 @@
         <v>185</v>
       </c>
       <c r="L67" s="5" t="s">
-        <v>250</v>
+        <v>206</v>
       </c>
       <c r="M67" s="5" t="s">
-        <v>251</v>
+        <v>441</v>
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">
@@ -4868,7 +4868,7 @@
         <v>147</v>
       </c>
       <c r="M68" s="5" t="s">
-        <v>252</v>
+        <v>442</v>
       </c>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
@@ -4909,7 +4909,7 @@
         <v>103</v>
       </c>
       <c r="M69" s="5" t="s">
-        <v>253</v>
+        <v>443</v>
       </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
@@ -4950,7 +4950,7 @@
         <v>137</v>
       </c>
       <c r="M70" s="5" t="s">
-        <v>254</v>
+        <v>444</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.25">
@@ -4991,7 +4991,7 @@
         <v>68</v>
       </c>
       <c r="M71" s="5" t="s">
-        <v>255</v>
+        <v>445</v>
       </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
@@ -5032,7 +5032,7 @@
         <v>68</v>
       </c>
       <c r="M72" s="5" t="s">
-        <v>256</v>
+        <v>446</v>
       </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
@@ -5073,7 +5073,7 @@
         <v>68</v>
       </c>
       <c r="M73" s="5" t="s">
-        <v>257</v>
+        <v>447</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
@@ -5102,19 +5102,19 @@
         <v>4710201197</v>
       </c>
       <c r="I74" s="5" t="s">
-        <v>258</v>
+        <v>207</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>259</v>
+        <v>208</v>
       </c>
       <c r="K74" s="5" t="s">
         <v>186</v>
       </c>
       <c r="L74" s="5" t="s">
-        <v>260</v>
+        <v>209</v>
       </c>
       <c r="M74" s="5" t="s">
-        <v>261</v>
+        <v>448</v>
       </c>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
@@ -5143,19 +5143,19 @@
         <v>4710201155</v>
       </c>
       <c r="I75" s="5" t="s">
-        <v>258</v>
+        <v>207</v>
       </c>
       <c r="J75" s="5" t="s">
-        <v>259</v>
+        <v>208</v>
       </c>
       <c r="K75" s="5" t="s">
         <v>186</v>
       </c>
       <c r="L75" s="5" t="s">
-        <v>260</v>
+        <v>209</v>
       </c>
       <c r="M75" s="5" t="s">
-        <v>262</v>
+        <v>449</v>
       </c>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.25">
@@ -5196,7 +5196,7 @@
         <v>157</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>263</v>
+        <v>450</v>
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.25">
@@ -5237,7 +5237,7 @@
         <v>33</v>
       </c>
       <c r="M77" s="5" t="s">
-        <v>264</v>
+        <v>451</v>
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.25">
@@ -5278,7 +5278,7 @@
         <v>160</v>
       </c>
       <c r="M78" s="5" t="s">
-        <v>265</v>
+        <v>452</v>
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
@@ -5319,7 +5319,7 @@
         <v>41</v>
       </c>
       <c r="M79" s="5" t="s">
-        <v>266</v>
+        <v>453</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.25">
@@ -5360,7 +5360,7 @@
         <v>163</v>
       </c>
       <c r="M80" s="5" t="s">
-        <v>267</v>
+        <v>454</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.25">
@@ -5401,7 +5401,7 @@
         <v>550</v>
       </c>
       <c r="M81" s="5" t="s">
-        <v>268</v>
+        <v>455</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.25">
@@ -5442,7 +5442,7 @@
         <v>166</v>
       </c>
       <c r="M82" s="5" t="s">
-        <v>269</v>
+        <v>456</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>33</v>
       </c>
       <c r="M83" s="5" t="s">
-        <v>270</v>
+        <v>457</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.25">
@@ -5524,7 +5524,7 @@
         <v>172</v>
       </c>
       <c r="M84" s="5" t="s">
-        <v>271</v>
+        <v>458</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.25">
@@ -5565,7 +5565,7 @@
         <v>41</v>
       </c>
       <c r="M85" s="5" t="s">
-        <v>272</v>
+        <v>459</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.25">
@@ -5606,7 +5606,7 @@
         <v>173</v>
       </c>
       <c r="M86" s="5" t="s">
-        <v>273</v>
+        <v>460</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.25">
@@ -5647,7 +5647,7 @@
         <v>175</v>
       </c>
       <c r="M87" s="5" t="s">
-        <v>274</v>
+        <v>461</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.25">
@@ -5676,7 +5676,7 @@
         <v>4712001379</v>
       </c>
       <c r="I88" s="5" t="s">
-        <v>275</v>
+        <v>210</v>
       </c>
       <c r="J88" s="5" t="s">
         <v>37</v>
@@ -5688,7 +5688,7 @@
         <v>600</v>
       </c>
       <c r="M88" s="5" t="s">
-        <v>276</v>
+        <v>462</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.25">
@@ -5729,7 +5729,7 @@
         <v>163</v>
       </c>
       <c r="M89" s="5" t="s">
-        <v>277</v>
+        <v>463</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.25">
@@ -5770,7 +5770,7 @@
         <v>126</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>278</v>
+        <v>464</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.25">
@@ -5811,7 +5811,7 @@
         <v>41</v>
       </c>
       <c r="M91" s="5" t="s">
-        <v>279</v>
+        <v>465</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.25">
@@ -5852,7 +5852,7 @@
         <v>170</v>
       </c>
       <c r="M92" s="5" t="s">
-        <v>280</v>
+        <v>466</v>
       </c>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.25">
@@ -5881,7 +5881,7 @@
         <v>4711200727</v>
       </c>
       <c r="I93" s="5" t="s">
-        <v>281</v>
+        <v>211</v>
       </c>
       <c r="J93" s="5" t="s">
         <v>37</v>
@@ -5890,10 +5890,10 @@
         <v>185</v>
       </c>
       <c r="L93" s="5" t="s">
-        <v>282</v>
+        <v>212</v>
       </c>
       <c r="M93" s="5" t="s">
-        <v>283</v>
+        <v>467</v>
       </c>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.25">
@@ -5922,7 +5922,7 @@
         <v>4712002037</v>
       </c>
       <c r="I94" s="5" t="s">
-        <v>284</v>
+        <v>213</v>
       </c>
       <c r="J94" s="5" t="s">
         <v>37</v>
@@ -5931,10 +5931,10 @@
         <v>185</v>
       </c>
       <c r="L94" s="5" t="s">
-        <v>285</v>
+        <v>214</v>
       </c>
       <c r="M94" s="5" t="s">
-        <v>286</v>
+        <v>468</v>
       </c>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.25">
@@ -5969,13 +5969,13 @@
         <v>180</v>
       </c>
       <c r="K95" s="5" t="s">
-        <v>287</v>
+        <v>215</v>
       </c>
       <c r="L95" s="5" t="s">
         <v>181</v>
       </c>
       <c r="M95" s="5" t="s">
-        <v>288</v>
+        <v>469</v>
       </c>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.25">
@@ -6004,10 +6004,10 @@
         <v>4711201805</v>
       </c>
       <c r="I96" s="5" t="s">
-        <v>289</v>
+        <v>216</v>
       </c>
       <c r="J96" s="5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K96" s="5" t="s">
         <v>186</v>
@@ -6016,7 +6016,7 @@
         <v>147</v>
       </c>
       <c r="M96" s="5" t="s">
-        <v>290</v>
+        <v>470</v>
       </c>
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.25">
@@ -6057,7 +6057,7 @@
         <v>68</v>
       </c>
       <c r="M97" s="5" t="s">
-        <v>291</v>
+        <v>471</v>
       </c>
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.25">
@@ -6098,7 +6098,7 @@
         <v>143</v>
       </c>
       <c r="M98" s="5" t="s">
-        <v>292</v>
+        <v>472</v>
       </c>
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.25">
@@ -6127,7 +6127,7 @@
         <v>4729105131</v>
       </c>
       <c r="I99" s="5" t="s">
-        <v>293</v>
+        <v>217</v>
       </c>
       <c r="J99" s="5" t="s">
         <v>37</v>
@@ -6136,10 +6136,10 @@
         <v>185</v>
       </c>
       <c r="L99" s="5" t="s">
-        <v>294</v>
+        <v>218</v>
       </c>
       <c r="M99" s="5" t="s">
-        <v>295</v>
+        <v>473</v>
       </c>
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.25">
@@ -6168,7 +6168,7 @@
         <v>4729105131</v>
       </c>
       <c r="I100" s="5" t="s">
-        <v>296</v>
+        <v>219</v>
       </c>
       <c r="J100" s="5" t="s">
         <v>37</v>
@@ -6180,7 +6180,7 @@
         <v>150</v>
       </c>
       <c r="M100" s="5" t="s">
-        <v>297</v>
+        <v>474</v>
       </c>
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.25">
@@ -6209,7 +6209,7 @@
         <v>4729105131</v>
       </c>
       <c r="I101" s="5" t="s">
-        <v>298</v>
+        <v>220</v>
       </c>
       <c r="J101" s="5" t="s">
         <v>37</v>
@@ -6218,18 +6218,18 @@
         <v>185</v>
       </c>
       <c r="L101" s="5" t="s">
-        <v>299</v>
+        <v>221</v>
       </c>
       <c r="M101" s="5" t="s">
-        <v>300</v>
+        <v>475</v>
       </c>
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>301</v>
+        <v>222</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C102" s="5">
         <v>14209967</v>
@@ -6250,7 +6250,7 @@
         <v>4710201184</v>
       </c>
       <c r="I102" s="5" t="s">
-        <v>303</v>
+        <v>224</v>
       </c>
       <c r="J102" s="5" t="s">
         <v>15</v>
@@ -6262,15 +6262,15 @@
         <v>160</v>
       </c>
       <c r="M102" s="5" t="s">
-        <v>304</v>
+        <v>476</v>
       </c>
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
-        <v>305</v>
+        <v>225</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C103" s="5">
         <v>14210518</v>
@@ -6291,7 +6291,7 @@
         <v>4711202059</v>
       </c>
       <c r="I103" s="5" t="s">
-        <v>306</v>
+        <v>226</v>
       </c>
       <c r="J103" s="5" t="s">
         <v>37</v>
@@ -6303,15 +6303,15 @@
         <v>360</v>
       </c>
       <c r="M103" s="5" t="s">
-        <v>307</v>
+        <v>477</v>
       </c>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>305</v>
+        <v>225</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C104" s="5">
         <v>14210621</v>
@@ -6332,7 +6332,7 @@
         <v>4718301283</v>
       </c>
       <c r="I104" s="5" t="s">
-        <v>308</v>
+        <v>227</v>
       </c>
       <c r="J104" s="5" t="s">
         <v>37</v>
@@ -6341,18 +6341,18 @@
         <v>185</v>
       </c>
       <c r="L104" s="5" t="s">
-        <v>309</v>
+        <v>228</v>
       </c>
       <c r="M104" s="5" t="s">
-        <v>310</v>
+        <v>478</v>
       </c>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
-        <v>305</v>
+        <v>225</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C105" s="5">
         <v>14210653</v>
@@ -6361,7 +6361,7 @@
         <v>14</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>311</v>
+        <v>479</v>
       </c>
       <c r="F105" s="5">
         <v>5</v>
@@ -6373,10 +6373,10 @@
         <v>4718300337</v>
       </c>
       <c r="I105" s="5" t="s">
-        <v>312</v>
+        <v>229</v>
       </c>
       <c r="J105" s="5" t="s">
-        <v>313</v>
+        <v>230</v>
       </c>
       <c r="K105" s="5" t="s">
         <v>186</v>
@@ -6385,15 +6385,15 @@
         <v>166</v>
       </c>
       <c r="M105" s="5" t="s">
-        <v>314</v>
+        <v>480</v>
       </c>
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>305</v>
+        <v>225</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C106" s="5">
         <v>14210666</v>
@@ -6411,10 +6411,10 @@
         <v>2</v>
       </c>
       <c r="H106" s="5" t="s">
-        <v>315</v>
+        <v>231</v>
       </c>
       <c r="I106" s="5" t="s">
-        <v>316</v>
+        <v>232</v>
       </c>
       <c r="J106" s="5" t="s">
         <v>37</v>
@@ -6426,15 +6426,15 @@
         <v>143</v>
       </c>
       <c r="M106" s="5" t="s">
-        <v>317</v>
+        <v>481</v>
       </c>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
-        <v>305</v>
+        <v>225</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C107" s="5">
         <v>14210666</v>
@@ -6452,10 +6452,10 @@
         <v>5</v>
       </c>
       <c r="H107" s="5" t="s">
-        <v>318</v>
+        <v>233</v>
       </c>
       <c r="I107" s="5" t="s">
-        <v>319</v>
+        <v>234</v>
       </c>
       <c r="J107" s="5" t="s">
         <v>37</v>
@@ -6464,18 +6464,18 @@
         <v>185</v>
       </c>
       <c r="L107" s="5" t="s">
-        <v>320</v>
+        <v>235</v>
       </c>
       <c r="M107" s="5" t="s">
-        <v>321</v>
+        <v>482</v>
       </c>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>305</v>
+        <v>225</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C108" s="5">
         <v>14210794</v>
@@ -6496,7 +6496,7 @@
         <v>4729110120</v>
       </c>
       <c r="I108" s="5" t="s">
-        <v>322</v>
+        <v>236</v>
       </c>
       <c r="J108" s="5" t="s">
         <v>37</v>
@@ -6508,15 +6508,15 @@
         <v>820</v>
       </c>
       <c r="M108" s="5" t="s">
-        <v>323</v>
+        <v>483</v>
       </c>
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C109" s="5">
         <v>14211272</v>
@@ -6534,10 +6534,10 @@
         <v>10</v>
       </c>
       <c r="H109" s="5" t="s">
-        <v>325</v>
+        <v>238</v>
       </c>
       <c r="I109" s="5" t="s">
-        <v>326</v>
+        <v>239</v>
       </c>
       <c r="J109" s="5" t="s">
         <v>37</v>
@@ -6549,15 +6549,15 @@
         <v>126</v>
       </c>
       <c r="M109" s="5" t="s">
-        <v>327</v>
+        <v>484</v>
       </c>
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C110" s="5">
         <v>14211388</v>
@@ -6578,7 +6578,7 @@
         <v>4711400231</v>
       </c>
       <c r="I110" s="5" t="s">
-        <v>328</v>
+        <v>240</v>
       </c>
       <c r="J110" s="5" t="s">
         <v>37</v>
@@ -6587,18 +6587,18 @@
         <v>185</v>
       </c>
       <c r="L110" s="5" t="s">
-        <v>282</v>
+        <v>212</v>
       </c>
       <c r="M110" s="5" t="s">
-        <v>329</v>
+        <v>485</v>
       </c>
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C111" s="5">
         <v>14211404</v>
@@ -6619,7 +6619,7 @@
         <v>4711400931</v>
       </c>
       <c r="I111" s="5" t="s">
-        <v>330</v>
+        <v>241</v>
       </c>
       <c r="J111" s="5" t="s">
         <v>50</v>
@@ -6628,18 +6628,18 @@
         <v>185</v>
       </c>
       <c r="L111" s="5" t="s">
-        <v>331</v>
+        <v>242</v>
       </c>
       <c r="M111" s="5" t="s">
-        <v>332</v>
+        <v>486</v>
       </c>
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C112" s="5">
         <v>14211411</v>
@@ -6660,7 +6660,7 @@
         <v>4729109063</v>
       </c>
       <c r="I112" s="5" t="s">
-        <v>333</v>
+        <v>243</v>
       </c>
       <c r="J112" s="5" t="s">
         <v>50</v>
@@ -6669,18 +6669,18 @@
         <v>185</v>
       </c>
       <c r="L112" s="5" t="s">
-        <v>334</v>
+        <v>244</v>
       </c>
       <c r="M112" s="5" t="s">
-        <v>335</v>
+        <v>487</v>
       </c>
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C113" s="5">
         <v>14211435</v>
@@ -6701,7 +6701,7 @@
         <v>4729401707</v>
       </c>
       <c r="I113" s="5" t="s">
-        <v>336</v>
+        <v>245</v>
       </c>
       <c r="J113" s="5" t="s">
         <v>50</v>
@@ -6713,15 +6713,15 @@
         <v>800</v>
       </c>
       <c r="M113" s="5" t="s">
-        <v>337</v>
+        <v>488</v>
       </c>
     </row>
     <row r="114" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C114" s="5">
         <v>14211440</v>
@@ -6754,15 +6754,15 @@
         <v>41</v>
       </c>
       <c r="M114" s="5" t="s">
-        <v>338</v>
+        <v>489</v>
       </c>
     </row>
     <row r="115" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C115" s="5">
         <v>14211447</v>
@@ -6795,15 +6795,15 @@
         <v>600</v>
       </c>
       <c r="M115" s="5" t="s">
-        <v>339</v>
+        <v>490</v>
       </c>
     </row>
     <row r="116" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C116" s="5">
         <v>14211453</v>
@@ -6821,30 +6821,30 @@
         <v>10</v>
       </c>
       <c r="H116" s="5" t="s">
-        <v>340</v>
+        <v>246</v>
       </c>
       <c r="I116" s="5" t="s">
-        <v>341</v>
+        <v>247</v>
       </c>
       <c r="J116" s="5" t="s">
-        <v>342</v>
+        <v>248</v>
       </c>
       <c r="K116" s="5" t="s">
-        <v>343</v>
+        <v>249</v>
       </c>
       <c r="L116" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M116" s="5" t="s">
-        <v>344</v>
+        <v>491</v>
       </c>
     </row>
     <row r="117" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C117" s="5">
         <v>14211457</v>
@@ -6877,15 +6877,15 @@
         <v>600</v>
       </c>
       <c r="M117" s="5" t="s">
-        <v>345</v>
+        <v>492</v>
       </c>
     </row>
     <row r="118" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C118" s="5">
         <v>14211459</v>
@@ -6918,15 +6918,15 @@
         <v>600</v>
       </c>
       <c r="M118" s="5" t="s">
-        <v>346</v>
+        <v>493</v>
       </c>
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C119" s="5">
         <v>14211464</v>
@@ -6959,15 +6959,15 @@
         <v>59</v>
       </c>
       <c r="M119" s="5" t="s">
-        <v>347</v>
+        <v>494</v>
       </c>
     </row>
     <row r="120" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C120" s="5">
         <v>14211477</v>
@@ -6988,7 +6988,7 @@
         <v>4729105685</v>
       </c>
       <c r="I120" s="5" t="s">
-        <v>348</v>
+        <v>250</v>
       </c>
       <c r="J120" s="5" t="s">
         <v>50</v>
@@ -7000,15 +7000,15 @@
         <v>430</v>
       </c>
       <c r="M120" s="5" t="s">
-        <v>349</v>
+        <v>495</v>
       </c>
     </row>
     <row r="121" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C121" s="5">
         <v>14211509</v>
@@ -7029,7 +7029,7 @@
         <v>4710101503</v>
       </c>
       <c r="I121" s="5" t="s">
-        <v>350</v>
+        <v>251</v>
       </c>
       <c r="J121" s="5" t="s">
         <v>37</v>
@@ -7038,18 +7038,18 @@
         <v>185</v>
       </c>
       <c r="L121" s="5" t="s">
-        <v>351</v>
+        <v>252</v>
       </c>
       <c r="M121" s="5" t="s">
-        <v>352</v>
+        <v>496</v>
       </c>
     </row>
     <row r="122" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C122" s="5">
         <v>14211553</v>
@@ -7070,7 +7070,7 @@
         <v>4304800227</v>
       </c>
       <c r="I122" s="5" t="s">
-        <v>353</v>
+        <v>253</v>
       </c>
       <c r="J122" s="5" t="s">
         <v>37</v>
@@ -7082,15 +7082,15 @@
         <v>110</v>
       </c>
       <c r="M122" s="5" t="s">
-        <v>354</v>
+        <v>497</v>
       </c>
     </row>
     <row r="123" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C123" s="5">
         <v>14211553</v>
@@ -7111,7 +7111,7 @@
         <v>4304800253</v>
       </c>
       <c r="I123" s="5" t="s">
-        <v>353</v>
+        <v>253</v>
       </c>
       <c r="J123" s="5" t="s">
         <v>37</v>
@@ -7123,15 +7123,15 @@
         <v>220</v>
       </c>
       <c r="M123" s="5" t="s">
-        <v>355</v>
+        <v>498</v>
       </c>
     </row>
     <row r="124" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C124" s="5">
         <v>14211553</v>
@@ -7152,7 +7152,7 @@
         <v>4304800229</v>
       </c>
       <c r="I124" s="5" t="s">
-        <v>353</v>
+        <v>253</v>
       </c>
       <c r="J124" s="5" t="s">
         <v>37</v>
@@ -7164,15 +7164,15 @@
         <v>550</v>
       </c>
       <c r="M124" s="5" t="s">
-        <v>356</v>
+        <v>499</v>
       </c>
     </row>
     <row r="125" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C125" s="5">
         <v>14211553</v>
@@ -7193,7 +7193,7 @@
         <v>4304800230</v>
       </c>
       <c r="I125" s="5" t="s">
-        <v>353</v>
+        <v>253</v>
       </c>
       <c r="J125" s="5" t="s">
         <v>37</v>
@@ -7205,15 +7205,15 @@
         <v>550</v>
       </c>
       <c r="M125" s="5" t="s">
-        <v>357</v>
+        <v>500</v>
       </c>
     </row>
     <row r="126" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C126" s="5">
         <v>14211553</v>
@@ -7234,7 +7234,7 @@
         <v>4719266003</v>
       </c>
       <c r="I126" s="5" t="s">
-        <v>353</v>
+        <v>253</v>
       </c>
       <c r="J126" s="5" t="s">
         <v>37</v>
@@ -7246,15 +7246,15 @@
         <v>110</v>
       </c>
       <c r="M126" s="5" t="s">
-        <v>358</v>
+        <v>501</v>
       </c>
     </row>
     <row r="127" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C127" s="5">
         <v>14211553</v>
@@ -7275,7 +7275,7 @@
         <v>4719266046</v>
       </c>
       <c r="I127" s="5" t="s">
-        <v>353</v>
+        <v>253</v>
       </c>
       <c r="J127" s="5" t="s">
         <v>37</v>
@@ -7287,15 +7287,15 @@
         <v>110</v>
       </c>
       <c r="M127" s="5" t="s">
-        <v>359</v>
+        <v>502</v>
       </c>
     </row>
     <row r="128" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>324</v>
+        <v>237</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C128" s="5">
         <v>14211575</v>
@@ -7313,10 +7313,10 @@
         <v>2</v>
       </c>
       <c r="H128" s="5" t="s">
-        <v>360</v>
+        <v>254</v>
       </c>
       <c r="I128" s="5" t="s">
-        <v>361</v>
+        <v>255</v>
       </c>
       <c r="J128" s="5" t="s">
         <v>37</v>
@@ -7328,15 +7328,15 @@
         <v>680</v>
       </c>
       <c r="M128" s="5" t="s">
-        <v>362</v>
+        <v>503</v>
       </c>
     </row>
     <row r="129" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C129" s="5">
         <v>14212112</v>
@@ -7357,7 +7357,7 @@
         <v>4712003208</v>
       </c>
       <c r="I129" s="5" t="s">
-        <v>364</v>
+        <v>257</v>
       </c>
       <c r="J129" s="5" t="s">
         <v>37</v>
@@ -7366,18 +7366,18 @@
         <v>185</v>
       </c>
       <c r="L129" s="5" t="s">
-        <v>365</v>
+        <v>258</v>
       </c>
       <c r="M129" s="5" t="s">
-        <v>366</v>
+        <v>504</v>
       </c>
     </row>
     <row r="130" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C130" s="5">
         <v>14212120</v>
@@ -7398,7 +7398,7 @@
         <v>4712004263</v>
       </c>
       <c r="I130" s="5" t="s">
-        <v>367</v>
+        <v>259</v>
       </c>
       <c r="J130" s="5" t="s">
         <v>37</v>
@@ -7410,15 +7410,15 @@
         <v>173</v>
       </c>
       <c r="M130" s="5" t="s">
-        <v>368</v>
+        <v>505</v>
       </c>
     </row>
     <row r="131" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C131" s="5">
         <v>14212124</v>
@@ -7439,27 +7439,27 @@
         <v>4711300621</v>
       </c>
       <c r="I131" s="5" t="s">
-        <v>369</v>
+        <v>260</v>
       </c>
       <c r="J131" s="5" t="s">
-        <v>370</v>
+        <v>261</v>
       </c>
       <c r="K131" s="5" t="s">
-        <v>371</v>
+        <v>262</v>
       </c>
       <c r="L131" s="5" t="s">
-        <v>372</v>
+        <v>263</v>
       </c>
       <c r="M131" s="5" t="s">
-        <v>373</v>
+        <v>506</v>
       </c>
     </row>
     <row r="132" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C132" s="5">
         <v>14212124</v>
@@ -7480,27 +7480,27 @@
         <v>4711300387</v>
       </c>
       <c r="I132" s="5" t="s">
-        <v>369</v>
+        <v>260</v>
       </c>
       <c r="J132" s="5" t="s">
-        <v>370</v>
+        <v>261</v>
       </c>
       <c r="K132" s="5" t="s">
-        <v>371</v>
+        <v>262</v>
       </c>
       <c r="L132" s="5" t="s">
-        <v>374</v>
+        <v>264</v>
       </c>
       <c r="M132" s="5" t="s">
-        <v>375</v>
+        <v>507</v>
       </c>
     </row>
     <row r="133" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C133" s="5">
         <v>14212245</v>
@@ -7521,7 +7521,7 @@
         <v>4712004409</v>
       </c>
       <c r="I133" s="5" t="s">
-        <v>376</v>
+        <v>265</v>
       </c>
       <c r="J133" s="5" t="s">
         <v>37</v>
@@ -7530,18 +7530,18 @@
         <v>185</v>
       </c>
       <c r="L133" s="5" t="s">
-        <v>365</v>
+        <v>258</v>
       </c>
       <c r="M133" s="5" t="s">
-        <v>377</v>
+        <v>508</v>
       </c>
     </row>
     <row r="134" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C134" s="5">
         <v>14212245</v>
@@ -7562,7 +7562,7 @@
         <v>4712004594</v>
       </c>
       <c r="I134" s="5" t="s">
-        <v>378</v>
+        <v>266</v>
       </c>
       <c r="J134" s="5" t="s">
         <v>37</v>
@@ -7571,18 +7571,18 @@
         <v>185</v>
       </c>
       <c r="L134" s="5" t="s">
-        <v>365</v>
+        <v>258</v>
       </c>
       <c r="M134" s="5" t="s">
-        <v>379</v>
+        <v>509</v>
       </c>
     </row>
     <row r="135" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C135" s="5">
         <v>14212254</v>
@@ -7600,10 +7600,10 @@
         <v>1</v>
       </c>
       <c r="H135" s="5" t="s">
-        <v>380</v>
+        <v>267</v>
       </c>
       <c r="I135" s="5" t="s">
-        <v>381</v>
+        <v>268</v>
       </c>
       <c r="J135" s="5" t="s">
         <v>37</v>
@@ -7612,18 +7612,18 @@
         <v>185</v>
       </c>
       <c r="L135" s="5" t="s">
-        <v>382</v>
+        <v>269</v>
       </c>
       <c r="M135" s="5" t="s">
-        <v>383</v>
+        <v>510</v>
       </c>
     </row>
     <row r="136" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>363</v>
+        <v>256</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C136" s="5">
         <v>14212254</v>
@@ -7641,10 +7641,10 @@
         <v>1</v>
       </c>
       <c r="H136" s="5" t="s">
-        <v>384</v>
+        <v>270</v>
       </c>
       <c r="I136" s="5" t="s">
-        <v>385</v>
+        <v>271</v>
       </c>
       <c r="J136" s="5" t="s">
         <v>37</v>
@@ -7656,15 +7656,15 @@
         <v>250</v>
       </c>
       <c r="M136" s="5" t="s">
-        <v>386</v>
+        <v>511</v>
       </c>
     </row>
     <row r="137" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C137" s="5">
         <v>14212686</v>
@@ -7682,10 +7682,10 @@
         <v>10</v>
       </c>
       <c r="H137" s="5" t="s">
-        <v>388</v>
+        <v>273</v>
       </c>
       <c r="I137" s="5" t="s">
-        <v>389</v>
+        <v>274</v>
       </c>
       <c r="J137" s="5" t="s">
         <v>37</v>
@@ -7697,15 +7697,15 @@
         <v>157</v>
       </c>
       <c r="M137" s="5" t="s">
-        <v>390</v>
+        <v>512</v>
       </c>
     </row>
     <row r="138" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C138" s="5">
         <v>14212761</v>
@@ -7726,7 +7726,7 @@
         <v>4702500847</v>
       </c>
       <c r="I138" s="5" t="s">
-        <v>391</v>
+        <v>275</v>
       </c>
       <c r="J138" s="5" t="s">
         <v>37</v>
@@ -7738,15 +7738,15 @@
         <v>110</v>
       </c>
       <c r="M138" s="5" t="s">
-        <v>392</v>
+        <v>513</v>
       </c>
     </row>
     <row r="139" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C139" s="5">
         <v>14212761</v>
@@ -7767,7 +7767,7 @@
         <v>4702500848</v>
       </c>
       <c r="I139" s="5" t="s">
-        <v>393</v>
+        <v>276</v>
       </c>
       <c r="J139" s="5" t="s">
         <v>37</v>
@@ -7779,15 +7779,15 @@
         <v>19</v>
       </c>
       <c r="M139" s="5" t="s">
-        <v>394</v>
+        <v>514</v>
       </c>
     </row>
     <row r="140" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C140" s="5">
         <v>14212803</v>
@@ -7808,7 +7808,7 @@
         <v>4711401085</v>
       </c>
       <c r="I140" s="5" t="s">
-        <v>395</v>
+        <v>277</v>
       </c>
       <c r="J140" s="5" t="s">
         <v>37</v>
@@ -7817,18 +7817,18 @@
         <v>185</v>
       </c>
       <c r="L140" s="5" t="s">
-        <v>396</v>
+        <v>278</v>
       </c>
       <c r="M140" s="5" t="s">
-        <v>397</v>
+        <v>515</v>
       </c>
     </row>
     <row r="141" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C141" s="5">
         <v>14212853</v>
@@ -7849,7 +7849,7 @@
         <v>4727501921</v>
       </c>
       <c r="I141" s="5" t="s">
-        <v>398</v>
+        <v>279</v>
       </c>
       <c r="J141" s="5" t="s">
         <v>50</v>
@@ -7861,15 +7861,15 @@
         <v>19</v>
       </c>
       <c r="M141" s="5" t="s">
-        <v>399</v>
+        <v>516</v>
       </c>
     </row>
     <row r="142" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C142" s="5">
         <v>14212865</v>
@@ -7890,7 +7890,7 @@
         <v>4712004670</v>
       </c>
       <c r="I142" s="5" t="s">
-        <v>400</v>
+        <v>280</v>
       </c>
       <c r="J142" s="5" t="s">
         <v>50</v>
@@ -7899,18 +7899,18 @@
         <v>185</v>
       </c>
       <c r="L142" s="5" t="s">
-        <v>401</v>
+        <v>281</v>
       </c>
       <c r="M142" s="5" t="s">
-        <v>402</v>
+        <v>517</v>
       </c>
     </row>
     <row r="143" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A143" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C143" s="5">
         <v>14212876</v>
@@ -7931,7 +7931,7 @@
         <v>4730502874</v>
       </c>
       <c r="I143" s="5" t="s">
-        <v>403</v>
+        <v>282</v>
       </c>
       <c r="J143" s="5" t="s">
         <v>37</v>
@@ -7943,15 +7943,15 @@
         <v>880</v>
       </c>
       <c r="M143" s="5" t="s">
-        <v>404</v>
+        <v>518</v>
       </c>
     </row>
     <row r="144" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C144" s="5">
         <v>14212949</v>
@@ -7972,7 +7972,7 @@
         <v>4729109250</v>
       </c>
       <c r="I144" s="5" t="s">
-        <v>405</v>
+        <v>283</v>
       </c>
       <c r="J144" s="5" t="s">
         <v>37</v>
@@ -7981,18 +7981,18 @@
         <v>185</v>
       </c>
       <c r="L144" s="5" t="s">
-        <v>406</v>
+        <v>284</v>
       </c>
       <c r="M144" s="5" t="s">
-        <v>407</v>
+        <v>519</v>
       </c>
     </row>
     <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C145" s="5">
         <v>14212952</v>
@@ -8013,7 +8013,7 @@
         <v>4730502878</v>
       </c>
       <c r="I145" s="5" t="s">
-        <v>408</v>
+        <v>285</v>
       </c>
       <c r="J145" s="5" t="s">
         <v>37</v>
@@ -8025,15 +8025,15 @@
         <v>650</v>
       </c>
       <c r="M145" s="5" t="s">
-        <v>409</v>
+        <v>520</v>
       </c>
     </row>
     <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C146" s="5">
         <v>14212953</v>
@@ -8054,7 +8054,7 @@
         <v>4727501154</v>
       </c>
       <c r="I146" s="5" t="s">
-        <v>410</v>
+        <v>286</v>
       </c>
       <c r="J146" s="5" t="s">
         <v>50</v>
@@ -8066,15 +8066,15 @@
         <v>800</v>
       </c>
       <c r="M146" s="5" t="s">
-        <v>411</v>
+        <v>521</v>
       </c>
     </row>
     <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C147" s="5">
         <v>14212955</v>
@@ -8095,7 +8095,7 @@
         <v>4711201791</v>
       </c>
       <c r="I147" s="5" t="s">
-        <v>412</v>
+        <v>287</v>
       </c>
       <c r="J147" s="5" t="s">
         <v>37</v>
@@ -8107,15 +8107,15 @@
         <v>173</v>
       </c>
       <c r="M147" s="5" t="s">
-        <v>413</v>
+        <v>522</v>
       </c>
     </row>
     <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C148" s="5">
         <v>14212957</v>
@@ -8136,7 +8136,7 @@
         <v>4727501155</v>
       </c>
       <c r="I148" s="5" t="s">
-        <v>410</v>
+        <v>286</v>
       </c>
       <c r="J148" s="5" t="s">
         <v>50</v>
@@ -8148,15 +8148,15 @@
         <v>400</v>
       </c>
       <c r="M148" s="5" t="s">
-        <v>414</v>
+        <v>523</v>
       </c>
     </row>
     <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C149" s="5">
         <v>14212962</v>
@@ -8189,15 +8189,15 @@
         <v>166</v>
       </c>
       <c r="M149" s="5" t="s">
-        <v>415</v>
+        <v>524</v>
       </c>
     </row>
     <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C150" s="5">
         <v>14212967</v>
@@ -8218,7 +8218,7 @@
         <v>4710101560</v>
       </c>
       <c r="I150" s="5" t="s">
-        <v>416</v>
+        <v>288</v>
       </c>
       <c r="J150" s="5" t="s">
         <v>37</v>
@@ -8230,15 +8230,15 @@
         <v>166</v>
       </c>
       <c r="M150" s="5" t="s">
-        <v>417</v>
+        <v>525</v>
       </c>
     </row>
     <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C151" s="5">
         <v>14212971</v>
@@ -8259,7 +8259,7 @@
         <v>4729108732</v>
       </c>
       <c r="I151" s="5" t="s">
-        <v>418</v>
+        <v>289</v>
       </c>
       <c r="J151" s="5" t="s">
         <v>37</v>
@@ -8271,15 +8271,15 @@
         <v>700</v>
       </c>
       <c r="M151" s="5" t="s">
-        <v>419</v>
+        <v>526</v>
       </c>
     </row>
     <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C152" s="5">
         <v>14213020</v>
@@ -8300,7 +8300,7 @@
         <v>4729110620</v>
       </c>
       <c r="I152" s="5" t="s">
-        <v>420</v>
+        <v>290</v>
       </c>
       <c r="J152" s="5" t="s">
         <v>37</v>
@@ -8312,15 +8312,15 @@
         <v>163</v>
       </c>
       <c r="M152" s="5" t="s">
-        <v>421</v>
+        <v>527</v>
       </c>
     </row>
     <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C153" s="5">
         <v>14213030</v>
@@ -8353,15 +8353,15 @@
         <v>166</v>
       </c>
       <c r="M153" s="5" t="s">
-        <v>422</v>
+        <v>528</v>
       </c>
     </row>
     <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C154" s="5">
         <v>14213034</v>
@@ -8394,15 +8394,15 @@
         <v>166</v>
       </c>
       <c r="M154" s="5" t="s">
-        <v>423</v>
+        <v>529</v>
       </c>
     </row>
     <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
-        <v>387</v>
+        <v>272</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C155" s="5">
         <v>14213104</v>
@@ -8420,30 +8420,30 @@
         <v>2</v>
       </c>
       <c r="H155" s="5" t="s">
-        <v>424</v>
+        <v>291</v>
       </c>
       <c r="I155" s="5" t="s">
-        <v>425</v>
+        <v>292</v>
       </c>
       <c r="J155" s="5" t="s">
-        <v>426</v>
+        <v>293</v>
       </c>
       <c r="K155" s="5" t="s">
-        <v>371</v>
+        <v>262</v>
       </c>
       <c r="L155" s="5" t="s">
         <v>103</v>
       </c>
       <c r="M155" s="5" t="s">
-        <v>427</v>
+        <v>530</v>
       </c>
     </row>
     <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="4" t="s">
-        <v>428</v>
+        <v>294</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C156" s="5">
         <v>14213297</v>
@@ -8464,7 +8464,7 @@
         <v>4727501151</v>
       </c>
       <c r="I156" s="5" t="s">
-        <v>429</v>
+        <v>295</v>
       </c>
       <c r="J156" s="5" t="s">
         <v>50</v>
@@ -8473,18 +8473,18 @@
         <v>185</v>
       </c>
       <c r="L156" s="5" t="s">
-        <v>430</v>
+        <v>296</v>
       </c>
       <c r="M156" s="5" t="s">
-        <v>431</v>
+        <v>531</v>
       </c>
     </row>
     <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
-        <v>428</v>
+        <v>294</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C157" s="5">
         <v>14213301</v>
@@ -8505,7 +8505,7 @@
         <v>4729104510</v>
       </c>
       <c r="I157" s="5" t="s">
-        <v>410</v>
+        <v>286</v>
       </c>
       <c r="J157" s="5" t="s">
         <v>50</v>
@@ -8514,18 +8514,18 @@
         <v>185</v>
       </c>
       <c r="L157" s="5" t="s">
-        <v>240</v>
+        <v>199</v>
       </c>
       <c r="M157" s="5" t="s">
-        <v>432</v>
+        <v>532</v>
       </c>
     </row>
     <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>428</v>
+        <v>294</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C158" s="5">
         <v>14213305</v>
@@ -8555,18 +8555,18 @@
         <v>185</v>
       </c>
       <c r="L158" s="5" t="s">
-        <v>433</v>
+        <v>297</v>
       </c>
       <c r="M158" s="5" t="s">
-        <v>434</v>
+        <v>533</v>
       </c>
     </row>
     <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="4" t="s">
-        <v>428</v>
+        <v>294</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C159" s="5">
         <v>14213308</v>
@@ -8587,7 +8587,7 @@
         <v>4711201528</v>
       </c>
       <c r="I159" s="5" t="s">
-        <v>435</v>
+        <v>298</v>
       </c>
       <c r="J159" s="5" t="s">
         <v>50</v>
@@ -8596,18 +8596,18 @@
         <v>185</v>
       </c>
       <c r="L159" s="5" t="s">
-        <v>436</v>
+        <v>299</v>
       </c>
       <c r="M159" s="5" t="s">
-        <v>437</v>
+        <v>534</v>
       </c>
     </row>
     <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="4" t="s">
-        <v>428</v>
+        <v>294</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C160" s="5">
         <v>14213310</v>
@@ -8628,7 +8628,7 @@
         <v>4712004047</v>
       </c>
       <c r="I160" s="5" t="s">
-        <v>438</v>
+        <v>300</v>
       </c>
       <c r="J160" s="5" t="s">
         <v>50</v>
@@ -8640,15 +8640,15 @@
         <v>68</v>
       </c>
       <c r="M160" s="5" t="s">
-        <v>439</v>
+        <v>535</v>
       </c>
     </row>
     <row r="161" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A161" s="4" t="s">
-        <v>428</v>
+        <v>294</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>302</v>
+        <v>223</v>
       </c>
       <c r="C161" s="5">
         <v>14213311</v>
@@ -8669,7 +8669,7 @@
         <v>4712004047</v>
       </c>
       <c r="I161" s="5" t="s">
-        <v>440</v>
+        <v>301</v>
       </c>
       <c r="J161" s="5" t="s">
         <v>50</v>
@@ -8681,15 +8681,15 @@
         <v>33</v>
       </c>
       <c r="M161" s="5" t="s">
-        <v>441</v>
+        <v>536</v>
       </c>
     </row>
     <row r="162" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A162" s="4" t="s">
-        <v>442</v>
+        <v>302</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C162" s="5">
         <v>14213659</v>
@@ -8710,7 +8710,7 @@
         <v>4710800192</v>
       </c>
       <c r="I162" s="5" t="s">
-        <v>444</v>
+        <v>304</v>
       </c>
       <c r="J162" s="5" t="s">
         <v>37</v>
@@ -8722,15 +8722,15 @@
         <v>112</v>
       </c>
       <c r="M162" s="5" t="s">
-        <v>445</v>
+        <v>305</v>
       </c>
     </row>
     <row r="163" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
-        <v>442</v>
+        <v>302</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C163" s="5">
         <v>14213659</v>
@@ -8763,15 +8763,15 @@
         <v>112</v>
       </c>
       <c r="M163" s="5" t="s">
-        <v>446</v>
+        <v>306</v>
       </c>
     </row>
     <row r="164" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A164" s="4" t="s">
-        <v>442</v>
+        <v>302</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C164" s="5">
         <v>14213693</v>
@@ -8792,7 +8792,7 @@
         <v>4729111555</v>
       </c>
       <c r="I164" s="5" t="s">
-        <v>447</v>
+        <v>307</v>
       </c>
       <c r="J164" s="5" t="s">
         <v>50</v>
@@ -8804,15 +8804,15 @@
         <v>38</v>
       </c>
       <c r="M164" s="5" t="s">
-        <v>448</v>
+        <v>308</v>
       </c>
     </row>
     <row r="165" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
-        <v>442</v>
+        <v>302</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C165" s="5">
         <v>14213876</v>
@@ -8833,7 +8833,7 @@
         <v>4728701223</v>
       </c>
       <c r="I165" s="5" t="s">
-        <v>449</v>
+        <v>309</v>
       </c>
       <c r="J165" s="5" t="s">
         <v>37</v>
@@ -8845,15 +8845,15 @@
         <v>880</v>
       </c>
       <c r="M165" s="5" t="s">
-        <v>450</v>
+        <v>310</v>
       </c>
     </row>
     <row r="166" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A166" s="4" t="s">
-        <v>442</v>
+        <v>302</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C166" s="5">
         <v>14213913</v>
@@ -8874,7 +8874,7 @@
         <v>4710201151</v>
       </c>
       <c r="I166" s="5" t="s">
-        <v>451</v>
+        <v>311</v>
       </c>
       <c r="J166" s="5" t="s">
         <v>37</v>
@@ -8883,18 +8883,18 @@
         <v>185</v>
       </c>
       <c r="L166" s="5" t="s">
-        <v>452</v>
+        <v>312</v>
       </c>
       <c r="M166" s="5" t="s">
-        <v>453</v>
+        <v>313</v>
       </c>
     </row>
     <row r="167" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A167" s="4" t="s">
-        <v>442</v>
+        <v>302</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C167" s="5">
         <v>14213936</v>
@@ -8915,7 +8915,7 @@
         <v>4729109958</v>
       </c>
       <c r="I167" s="5" t="s">
-        <v>454</v>
+        <v>314</v>
       </c>
       <c r="J167" s="5" t="s">
         <v>37</v>
@@ -8927,15 +8927,15 @@
         <v>59</v>
       </c>
       <c r="M167" s="5" t="s">
-        <v>455</v>
+        <v>315</v>
       </c>
     </row>
     <row r="168" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A168" s="4" t="s">
-        <v>442</v>
+        <v>302</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C168" s="5">
         <v>14213992</v>
@@ -8953,10 +8953,10 @@
         <v>4</v>
       </c>
       <c r="H168" s="5" t="s">
-        <v>456</v>
+        <v>316</v>
       </c>
       <c r="I168" s="5" t="s">
-        <v>457</v>
+        <v>317</v>
       </c>
       <c r="J168" s="5" t="s">
         <v>58</v>
@@ -8968,15 +8968,15 @@
         <v>800</v>
       </c>
       <c r="M168" s="5" t="s">
-        <v>458</v>
+        <v>318</v>
       </c>
     </row>
     <row r="169" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A169" s="4" t="s">
-        <v>459</v>
+        <v>319</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C169" s="5">
         <v>14214523</v>
@@ -8997,7 +8997,7 @@
         <v>4711202048</v>
       </c>
       <c r="I169" s="5" t="s">
-        <v>460</v>
+        <v>320</v>
       </c>
       <c r="J169" s="5" t="s">
         <v>37</v>
@@ -9009,15 +9009,15 @@
         <v>157</v>
       </c>
       <c r="M169" s="5" t="s">
-        <v>461</v>
+        <v>321</v>
       </c>
     </row>
     <row r="170" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A170" s="4" t="s">
-        <v>459</v>
+        <v>319</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C170" s="5">
         <v>14214728</v>
@@ -9038,7 +9038,7 @@
         <v>4728700283</v>
       </c>
       <c r="I170" s="5" t="s">
-        <v>462</v>
+        <v>322</v>
       </c>
       <c r="J170" s="5" t="s">
         <v>37</v>
@@ -9047,18 +9047,18 @@
         <v>185</v>
       </c>
       <c r="L170" s="5" t="s">
-        <v>463</v>
+        <v>323</v>
       </c>
       <c r="M170" s="5" t="s">
-        <v>464</v>
+        <v>324</v>
       </c>
     </row>
     <row r="171" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A171" s="4" t="s">
-        <v>459</v>
+        <v>319</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C171" s="5">
         <v>14214738</v>
@@ -9088,18 +9088,18 @@
         <v>185</v>
       </c>
       <c r="L171" s="5" t="s">
-        <v>465</v>
+        <v>325</v>
       </c>
       <c r="M171" s="5" t="s">
-        <v>466</v>
+        <v>326</v>
       </c>
     </row>
     <row r="172" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A172" s="4" t="s">
-        <v>459</v>
+        <v>319</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C172" s="5">
         <v>14214744</v>
@@ -9120,7 +9120,7 @@
         <v>4710101560</v>
       </c>
       <c r="I172" s="5" t="s">
-        <v>467</v>
+        <v>327</v>
       </c>
       <c r="J172" s="5" t="s">
         <v>37</v>
@@ -9132,15 +9132,15 @@
         <v>166</v>
       </c>
       <c r="M172" s="5" t="s">
-        <v>468</v>
+        <v>328</v>
       </c>
     </row>
     <row r="173" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A173" s="4" t="s">
-        <v>459</v>
+        <v>319</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C173" s="5">
         <v>14214825</v>
@@ -9161,7 +9161,7 @@
         <v>4727500865</v>
       </c>
       <c r="I173" s="5" t="s">
-        <v>469</v>
+        <v>329</v>
       </c>
       <c r="J173" s="5" t="s">
         <v>37</v>
@@ -9173,15 +9173,15 @@
         <v>114</v>
       </c>
       <c r="M173" s="5" t="s">
-        <v>470</v>
+        <v>330</v>
       </c>
     </row>
     <row r="174" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A174" s="4" t="s">
-        <v>471</v>
+        <v>331</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C174" s="5">
         <v>14215400</v>
@@ -9202,7 +9202,7 @@
         <v>4710101475</v>
       </c>
       <c r="I174" s="5" t="s">
-        <v>472</v>
+        <v>332</v>
       </c>
       <c r="J174" s="5" t="s">
         <v>37</v>
@@ -9211,18 +9211,18 @@
         <v>185</v>
       </c>
       <c r="L174" s="5" t="s">
-        <v>473</v>
+        <v>333</v>
       </c>
       <c r="M174" s="5" t="s">
-        <v>474</v>
+        <v>334</v>
       </c>
     </row>
     <row r="175" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A175" s="4" t="s">
-        <v>471</v>
+        <v>331</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C175" s="5">
         <v>14215433</v>
@@ -9240,30 +9240,30 @@
         <v>28</v>
       </c>
       <c r="H175" s="5" t="s">
-        <v>475</v>
+        <v>335</v>
       </c>
       <c r="I175" s="5" t="s">
-        <v>476</v>
+        <v>336</v>
       </c>
       <c r="J175" s="5" t="s">
-        <v>477</v>
+        <v>337</v>
       </c>
       <c r="K175" s="5" t="s">
-        <v>478</v>
+        <v>338</v>
       </c>
       <c r="L175" s="5" t="s">
-        <v>479</v>
+        <v>339</v>
       </c>
       <c r="M175" s="5" t="s">
-        <v>480</v>
+        <v>340</v>
       </c>
     </row>
     <row r="176" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A176" s="4" t="s">
-        <v>471</v>
+        <v>331</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C176" s="5">
         <v>14215504</v>
@@ -9296,15 +9296,15 @@
         <v>450</v>
       </c>
       <c r="M176" s="5" t="s">
-        <v>481</v>
+        <v>341</v>
       </c>
     </row>
     <row r="177" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A177" s="4" t="s">
-        <v>471</v>
+        <v>331</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C177" s="5">
         <v>14215675</v>
@@ -9325,27 +9325,27 @@
         <v>4711201529</v>
       </c>
       <c r="I177" s="5" t="s">
-        <v>482</v>
+        <v>342</v>
       </c>
       <c r="J177" s="5" t="s">
-        <v>483</v>
+        <v>343</v>
       </c>
       <c r="K177" s="5" t="s">
-        <v>484</v>
+        <v>344</v>
       </c>
       <c r="L177" s="5" t="s">
-        <v>485</v>
+        <v>345</v>
       </c>
       <c r="M177" s="5" t="s">
-        <v>486</v>
+        <v>346</v>
       </c>
     </row>
     <row r="178" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A178" s="4" t="s">
-        <v>487</v>
+        <v>347</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C178" s="5">
         <v>14216106</v>
@@ -9366,7 +9366,7 @@
         <v>4305400225</v>
       </c>
       <c r="I178" s="5" t="s">
-        <v>488</v>
+        <v>348</v>
       </c>
       <c r="J178" s="5" t="s">
         <v>37</v>
@@ -9378,15 +9378,15 @@
         <v>160</v>
       </c>
       <c r="M178" s="5" t="s">
-        <v>489</v>
+        <v>349</v>
       </c>
     </row>
     <row r="179" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A179" s="4" t="s">
-        <v>487</v>
+        <v>347</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C179" s="5">
         <v>14216222</v>
@@ -9407,7 +9407,7 @@
         <v>4729105785</v>
       </c>
       <c r="I179" s="5" t="s">
-        <v>490</v>
+        <v>350</v>
       </c>
       <c r="J179" s="5" t="s">
         <v>50</v>
@@ -9419,15 +9419,15 @@
         <v>68</v>
       </c>
       <c r="M179" s="5" t="s">
-        <v>491</v>
+        <v>351</v>
       </c>
     </row>
     <row r="180" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A180" s="4" t="s">
-        <v>487</v>
+        <v>347</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C180" s="5">
         <v>14216272</v>
@@ -9448,7 +9448,7 @@
         <v>4710800032</v>
       </c>
       <c r="I180" s="5" t="s">
-        <v>492</v>
+        <v>352</v>
       </c>
       <c r="J180" s="5" t="s">
         <v>37</v>
@@ -9460,15 +9460,15 @@
         <v>41</v>
       </c>
       <c r="M180" s="5" t="s">
-        <v>493</v>
+        <v>353</v>
       </c>
     </row>
     <row r="181" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A181" s="4" t="s">
-        <v>487</v>
+        <v>347</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C181" s="5">
         <v>14216272</v>
@@ -9489,7 +9489,7 @@
         <v>4710800002</v>
       </c>
       <c r="I181" s="5" t="s">
-        <v>492</v>
+        <v>352</v>
       </c>
       <c r="J181" s="5" t="s">
         <v>37</v>
@@ -9501,15 +9501,15 @@
         <v>173</v>
       </c>
       <c r="M181" s="5" t="s">
-        <v>494</v>
+        <v>354</v>
       </c>
     </row>
     <row r="182" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A182" s="4" t="s">
-        <v>487</v>
+        <v>347</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C182" s="5">
         <v>14216272</v>
@@ -9530,7 +9530,7 @@
         <v>4710800100</v>
       </c>
       <c r="I182" s="5" t="s">
-        <v>492</v>
+        <v>352</v>
       </c>
       <c r="J182" s="5" t="s">
         <v>37</v>
@@ -9542,15 +9542,15 @@
         <v>47</v>
       </c>
       <c r="M182" s="5" t="s">
-        <v>495</v>
+        <v>355</v>
       </c>
     </row>
     <row r="183" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A183" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C183" s="5">
         <v>14216678</v>
@@ -9571,7 +9571,7 @@
         <v>4729111741</v>
       </c>
       <c r="I183" s="5" t="s">
-        <v>497</v>
+        <v>357</v>
       </c>
       <c r="J183" s="5" t="s">
         <v>37</v>
@@ -9583,15 +9583,15 @@
         <v>143</v>
       </c>
       <c r="M183" s="5" t="s">
-        <v>498</v>
+        <v>358</v>
       </c>
     </row>
     <row r="184" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A184" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C184" s="5">
         <v>14216857</v>
@@ -9609,10 +9609,10 @@
         <v>2</v>
       </c>
       <c r="H184" s="5" t="s">
-        <v>499</v>
+        <v>359</v>
       </c>
       <c r="I184" s="5" t="s">
-        <v>500</v>
+        <v>360</v>
       </c>
       <c r="J184" s="5" t="s">
         <v>37</v>
@@ -9621,18 +9621,18 @@
         <v>185</v>
       </c>
       <c r="L184" s="5" t="s">
-        <v>501</v>
+        <v>361</v>
       </c>
       <c r="M184" s="5" t="s">
-        <v>502</v>
+        <v>362</v>
       </c>
     </row>
     <row r="185" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A185" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C185" s="5">
         <v>14216857</v>
@@ -9650,10 +9650,10 @@
         <v>2</v>
       </c>
       <c r="H185" s="5" t="s">
-        <v>503</v>
+        <v>363</v>
       </c>
       <c r="I185" s="5" t="s">
-        <v>504</v>
+        <v>364</v>
       </c>
       <c r="J185" s="5" t="s">
         <v>37</v>
@@ -9662,18 +9662,18 @@
         <v>185</v>
       </c>
       <c r="L185" s="5" t="s">
-        <v>501</v>
+        <v>361</v>
       </c>
       <c r="M185" s="5" t="s">
-        <v>505</v>
+        <v>365</v>
       </c>
     </row>
     <row r="186" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A186" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C186" s="5">
         <v>14216857</v>
@@ -9691,10 +9691,10 @@
         <v>2</v>
       </c>
       <c r="H186" s="5" t="s">
-        <v>506</v>
+        <v>366</v>
       </c>
       <c r="I186" s="5" t="s">
-        <v>507</v>
+        <v>367</v>
       </c>
       <c r="J186" s="5" t="s">
         <v>37</v>
@@ -9703,18 +9703,18 @@
         <v>185</v>
       </c>
       <c r="L186" s="5" t="s">
-        <v>501</v>
+        <v>361</v>
       </c>
       <c r="M186" s="5" t="s">
-        <v>508</v>
+        <v>368</v>
       </c>
     </row>
     <row r="187" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A187" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C187" s="5">
         <v>14216857</v>
@@ -9732,10 +9732,10 @@
         <v>2</v>
       </c>
       <c r="H187" s="5" t="s">
-        <v>509</v>
+        <v>369</v>
       </c>
       <c r="I187" s="5" t="s">
-        <v>510</v>
+        <v>370</v>
       </c>
       <c r="J187" s="5" t="s">
         <v>37</v>
@@ -9744,18 +9744,18 @@
         <v>185</v>
       </c>
       <c r="L187" s="5" t="s">
-        <v>511</v>
+        <v>371</v>
       </c>
       <c r="M187" s="5" t="s">
-        <v>512</v>
+        <v>372</v>
       </c>
     </row>
     <row r="188" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A188" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C188" s="5">
         <v>14216857</v>
@@ -9773,10 +9773,10 @@
         <v>2</v>
       </c>
       <c r="H188" s="5" t="s">
-        <v>513</v>
+        <v>373</v>
       </c>
       <c r="I188" s="5" t="s">
-        <v>514</v>
+        <v>374</v>
       </c>
       <c r="J188" s="5" t="s">
         <v>37</v>
@@ -9785,18 +9785,18 @@
         <v>185</v>
       </c>
       <c r="L188" s="5" t="s">
-        <v>511</v>
+        <v>371</v>
       </c>
       <c r="M188" s="5" t="s">
-        <v>515</v>
+        <v>375</v>
       </c>
     </row>
     <row r="189" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A189" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C189" s="5">
         <v>14216925</v>
@@ -9817,7 +9817,7 @@
         <v>4730502923</v>
       </c>
       <c r="I189" s="5" t="s">
-        <v>516</v>
+        <v>376</v>
       </c>
       <c r="J189" s="5" t="s">
         <v>50</v>
@@ -9829,15 +9829,15 @@
         <v>800</v>
       </c>
       <c r="M189" s="5" t="s">
-        <v>517</v>
+        <v>377</v>
       </c>
     </row>
     <row r="190" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A190" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C190" s="5">
         <v>14216965</v>
@@ -9858,7 +9858,7 @@
         <v>4729106006</v>
       </c>
       <c r="I190" s="5" t="s">
-        <v>518</v>
+        <v>378</v>
       </c>
       <c r="J190" s="5" t="s">
         <v>58</v>
@@ -9870,15 +9870,15 @@
         <v>157</v>
       </c>
       <c r="M190" s="5" t="s">
-        <v>519</v>
+        <v>379</v>
       </c>
     </row>
     <row r="191" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A191" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C191" s="5">
         <v>14216976</v>
@@ -9899,7 +9899,7 @@
         <v>4320600139</v>
       </c>
       <c r="I191" s="5" t="s">
-        <v>520</v>
+        <v>380</v>
       </c>
       <c r="J191" s="5" t="s">
         <v>37</v>
@@ -9908,18 +9908,18 @@
         <v>185</v>
       </c>
       <c r="L191" s="5" t="s">
-        <v>521</v>
+        <v>381</v>
       </c>
       <c r="M191" s="5" t="s">
-        <v>522</v>
+        <v>382</v>
       </c>
     </row>
     <row r="192" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A192" s="4" t="s">
-        <v>496</v>
+        <v>356</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>443</v>
+        <v>303</v>
       </c>
       <c r="C192" s="5">
         <v>14217041</v>
@@ -9940,7 +9940,7 @@
         <v>4729112103</v>
       </c>
       <c r="I192" s="5" t="s">
-        <v>523</v>
+        <v>383</v>
       </c>
       <c r="J192" s="5" t="s">
         <v>58</v>
@@ -9949,18 +9949,18 @@
         <v>185</v>
       </c>
       <c r="L192" s="5" t="s">
-        <v>524</v>
+        <v>384</v>
       </c>
       <c r="M192" s="5" t="s">
-        <v>525</v>
+        <v>385</v>
       </c>
     </row>
     <row r="193" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A193" s="4" t="s">
-        <v>526</v>
+        <v>386</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>527</v>
+        <v>387</v>
       </c>
       <c r="C193" s="5">
         <v>14217734</v>
@@ -9981,7 +9981,7 @@
         <v>4711401061</v>
       </c>
       <c r="I193" s="5" t="s">
-        <v>528</v>
+        <v>388</v>
       </c>
       <c r="J193" s="5" t="s">
         <v>58</v>
@@ -9990,18 +9990,18 @@
         <v>185</v>
       </c>
       <c r="L193" s="5" t="s">
-        <v>529</v>
+        <v>389</v>
       </c>
       <c r="M193" s="5" t="s">
-        <v>530</v>
+        <v>390</v>
       </c>
     </row>
     <row r="194" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A194" s="4" t="s">
-        <v>526</v>
+        <v>386</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>527</v>
+        <v>387</v>
       </c>
       <c r="C194" s="5">
         <v>14218303</v>
@@ -10022,7 +10022,7 @@
         <v>4712002707</v>
       </c>
       <c r="I194" s="5" t="s">
-        <v>523</v>
+        <v>383</v>
       </c>
       <c r="J194" s="5" t="s">
         <v>58</v>
@@ -10031,18 +10031,18 @@
         <v>185</v>
       </c>
       <c r="L194" s="5" t="s">
-        <v>531</v>
+        <v>391</v>
       </c>
       <c r="M194" s="5" t="s">
-        <v>532</v>
+        <v>392</v>
       </c>
     </row>
     <row r="195" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A195" s="4" t="s">
-        <v>526</v>
+        <v>386</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>527</v>
+        <v>387</v>
       </c>
       <c r="C195" s="5">
         <v>14218494</v>
@@ -10075,15 +10075,15 @@
         <v>600</v>
       </c>
       <c r="M195" s="5" t="s">
-        <v>533</v>
+        <v>393</v>
       </c>
     </row>
     <row r="196" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A196" s="4" t="s">
-        <v>526</v>
+        <v>386</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>527</v>
+        <v>387</v>
       </c>
       <c r="C196" s="5">
         <v>14218497</v>
@@ -10116,15 +10116,15 @@
         <v>600</v>
       </c>
       <c r="M196" s="5" t="s">
-        <v>534</v>
+        <v>394</v>
       </c>
     </row>
     <row r="197" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A197" s="4" t="s">
-        <v>526</v>
+        <v>386</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>527</v>
+        <v>387</v>
       </c>
       <c r="C197" s="5">
         <v>14218498</v>
@@ -10145,7 +10145,7 @@
         <v>4712003439</v>
       </c>
       <c r="I197" s="5" t="s">
-        <v>535</v>
+        <v>395</v>
       </c>
       <c r="J197" s="5" t="s">
         <v>58</v>
@@ -10157,7 +10157,7 @@
         <v>660</v>
       </c>
       <c r="M197" s="5" t="s">
-        <v>536</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used: lp register bot
</commit_message>
<xml_diff>
--- a/98 - Excels/Cadastro-LPs.xlsx
+++ b/98 - Excels/Cadastro-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feb3ct\Desktop\PyAutomateSAP\98 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14AE0472-A711-4BE0-8D09-62826A1578FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD9FBC2-E6A0-4E0F-9C87-C56D625C6829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2076" uniqueCount="643">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2182" uniqueCount="644">
   <si>
     <t>Data</t>
   </si>
@@ -1949,6 +1949,9 @@
   </si>
   <si>
     <t>LP-055834</t>
+  </si>
+  <si>
+    <t>CADASTRADA</t>
   </si>
 </sst>
 </file>
@@ -2456,7 +2459,9 @@
       <c r="M2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="N2" s="5"/>
+      <c r="N2" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O2" s="5"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -2499,7 +2504,9 @@
       <c r="M3" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="N3" s="5"/>
+      <c r="N3" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O3" s="5"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -2542,7 +2549,9 @@
       <c r="M4" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="N4" s="5"/>
+      <c r="N4" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -2585,7 +2594,9 @@
       <c r="M5" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="N5" s="5"/>
+      <c r="N5" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O5" s="5"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -2628,7 +2639,9 @@
       <c r="M6" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="5"/>
+      <c r="N6" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -2671,7 +2684,9 @@
       <c r="M7" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="N7" s="5"/>
+      <c r="N7" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O7" s="5"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -2714,7 +2729,9 @@
       <c r="M8" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="N8" s="5"/>
+      <c r="N8" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O8" s="5"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -2757,7 +2774,9 @@
       <c r="M9" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="N9" s="5"/>
+      <c r="N9" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O9" s="5"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -2800,7 +2819,9 @@
       <c r="M10" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="N10" s="5"/>
+      <c r="N10" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O10" s="5"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -2843,7 +2864,9 @@
       <c r="M11" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="N11" s="5"/>
+      <c r="N11" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O11" s="5"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2886,7 +2909,9 @@
       <c r="M12" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="N12" s="5"/>
+      <c r="N12" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O12" s="5"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -2929,7 +2954,9 @@
       <c r="M13" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="N13" s="5"/>
+      <c r="N13" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O13" s="5"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -2972,7 +2999,9 @@
       <c r="M14" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="N14" s="5"/>
+      <c r="N14" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O14" s="5"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -3015,7 +3044,9 @@
       <c r="M15" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="5"/>
+      <c r="N15" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O15" s="5"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -3058,7 +3089,9 @@
       <c r="M16" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="N16" s="5"/>
+      <c r="N16" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O16" s="5"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -3101,7 +3134,9 @@
       <c r="M17" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="N17" s="5"/>
+      <c r="N17" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O17" s="5"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -3144,7 +3179,9 @@
       <c r="M18" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="N18" s="5"/>
+      <c r="N18" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O18" s="5"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -3187,7 +3224,9 @@
       <c r="M19" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="N19" s="5"/>
+      <c r="N19" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O19" s="5"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -3230,7 +3269,9 @@
       <c r="M20" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="N20" s="5"/>
+      <c r="N20" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O20" s="5"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -3273,7 +3314,9 @@
       <c r="M21" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="N21" s="5"/>
+      <c r="N21" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O21" s="5"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -3316,7 +3359,9 @@
       <c r="M22" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="N22" s="5"/>
+      <c r="N22" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O22" s="5"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -3359,7 +3404,9 @@
       <c r="M23" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="N23" s="5"/>
+      <c r="N23" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O23" s="5"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -3402,7 +3449,9 @@
       <c r="M24" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="N24" s="5"/>
+      <c r="N24" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O24" s="5"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -3445,7 +3494,9 @@
       <c r="M25" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="N25" s="5"/>
+      <c r="N25" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O25" s="5"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -3488,7 +3539,9 @@
       <c r="M26" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="N26" s="5"/>
+      <c r="N26" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O26" s="5"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -3531,7 +3584,9 @@
       <c r="M27" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="N27" s="5"/>
+      <c r="N27" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O27" s="5"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -3574,7 +3629,9 @@
       <c r="M28" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="N28" s="5"/>
+      <c r="N28" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O28" s="5"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -3617,7 +3674,9 @@
       <c r="M29" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="N29" s="5"/>
+      <c r="N29" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O29" s="5"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -3660,7 +3719,9 @@
       <c r="M30" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="N30" s="5"/>
+      <c r="N30" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O30" s="5"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -3703,7 +3764,9 @@
       <c r="M31" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="N31" s="5"/>
+      <c r="N31" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O31" s="5"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -3746,7 +3809,9 @@
       <c r="M32" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="N32" s="5"/>
+      <c r="N32" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O32" s="5"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -3789,7 +3854,9 @@
       <c r="M33" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="N33" s="5"/>
+      <c r="N33" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O33" s="5"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
@@ -3832,7 +3899,9 @@
       <c r="M34" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="N34" s="5"/>
+      <c r="N34" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O34" s="5"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
@@ -3875,7 +3944,9 @@
       <c r="M35" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="N35" s="5"/>
+      <c r="N35" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O35" s="5"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
@@ -3918,7 +3989,9 @@
       <c r="M36" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="N36" s="5"/>
+      <c r="N36" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O36" s="5"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
@@ -3961,7 +4034,9 @@
       <c r="M37" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="N37" s="5"/>
+      <c r="N37" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O37" s="5"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
@@ -4004,7 +4079,9 @@
       <c r="M38" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="N38" s="5"/>
+      <c r="N38" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O38" s="5"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
@@ -4047,7 +4124,9 @@
       <c r="M39" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="N39" s="5"/>
+      <c r="N39" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O39" s="5"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
@@ -4090,7 +4169,9 @@
       <c r="M40" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="N40" s="5"/>
+      <c r="N40" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O40" s="5"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
@@ -4133,7 +4214,9 @@
       <c r="M41" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="N41" s="5"/>
+      <c r="N41" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O41" s="5"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
@@ -4176,7 +4259,9 @@
       <c r="M42" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="N42" s="5"/>
+      <c r="N42" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O42" s="5"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
@@ -4219,7 +4304,9 @@
       <c r="M43" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="N43" s="5"/>
+      <c r="N43" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O43" s="5"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
@@ -4262,7 +4349,9 @@
       <c r="M44" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="N44" s="5"/>
+      <c r="N44" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O44" s="5"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
@@ -4305,7 +4394,9 @@
       <c r="M45" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="N45" s="5"/>
+      <c r="N45" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O45" s="5"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
@@ -4348,7 +4439,9 @@
       <c r="M46" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="N46" s="5"/>
+      <c r="N46" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O46" s="5"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
@@ -4391,7 +4484,9 @@
       <c r="M47" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="N47" s="5"/>
+      <c r="N47" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O47" s="5"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
@@ -4434,7 +4529,9 @@
       <c r="M48" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="N48" s="5"/>
+      <c r="N48" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O48" s="5"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
@@ -4477,7 +4574,9 @@
       <c r="M49" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="N49" s="5"/>
+      <c r="N49" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O49" s="5"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
@@ -4520,7 +4619,9 @@
       <c r="M50" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="N50" s="5"/>
+      <c r="N50" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O50" s="5"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
@@ -4563,7 +4664,9 @@
       <c r="M51" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="N51" s="5"/>
+      <c r="N51" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O51" s="5"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
@@ -4606,7 +4709,9 @@
       <c r="M52" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="N52" s="5"/>
+      <c r="N52" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O52" s="5"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
@@ -4649,7 +4754,9 @@
       <c r="M53" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="N53" s="5"/>
+      <c r="N53" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O53" s="5"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
@@ -4692,7 +4799,9 @@
       <c r="M54" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="N54" s="5"/>
+      <c r="N54" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O54" s="5"/>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
@@ -4735,7 +4844,9 @@
       <c r="M55" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="N55" s="5"/>
+      <c r="N55" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O55" s="5"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
@@ -4778,7 +4889,9 @@
       <c r="M56" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="N56" s="5"/>
+      <c r="N56" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O56" s="5"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
@@ -4821,7 +4934,9 @@
       <c r="M57" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="N57" s="5"/>
+      <c r="N57" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O57" s="5"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
@@ -4864,7 +4979,9 @@
       <c r="M58" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="N58" s="5"/>
+      <c r="N58" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O58" s="5"/>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
@@ -4907,7 +5024,9 @@
       <c r="M59" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="N59" s="5"/>
+      <c r="N59" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O59" s="5"/>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
@@ -4950,7 +5069,9 @@
       <c r="M60" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="N60" s="5"/>
+      <c r="N60" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O60" s="5"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
@@ -4993,7 +5114,9 @@
       <c r="M61" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="N61" s="5"/>
+      <c r="N61" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O61" s="5"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
@@ -5036,7 +5159,9 @@
       <c r="M62" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="N62" s="5"/>
+      <c r="N62" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O62" s="5"/>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
@@ -5079,7 +5204,9 @@
       <c r="M63" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="N63" s="5"/>
+      <c r="N63" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O63" s="5"/>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
@@ -5122,7 +5249,9 @@
       <c r="M64" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="N64" s="5"/>
+      <c r="N64" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O64" s="5"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
@@ -5165,7 +5294,9 @@
       <c r="M65" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="N65" s="5"/>
+      <c r="N65" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O65" s="5"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
@@ -5208,7 +5339,9 @@
       <c r="M66" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="N66" s="5"/>
+      <c r="N66" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O66" s="5"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
@@ -5251,7 +5384,9 @@
       <c r="M67" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="N67" s="5"/>
+      <c r="N67" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O67" s="5"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
@@ -5294,7 +5429,9 @@
       <c r="M68" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="N68" s="5"/>
+      <c r="N68" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O68" s="5"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
@@ -5337,7 +5474,9 @@
       <c r="M69" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="N69" s="5"/>
+      <c r="N69" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O69" s="5"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
@@ -5380,7 +5519,9 @@
       <c r="M70" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="N70" s="5"/>
+      <c r="N70" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O70" s="5"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.25">
@@ -5423,7 +5564,9 @@
       <c r="M71" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="N71" s="5"/>
+      <c r="N71" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O71" s="5"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
@@ -5466,7 +5609,9 @@
       <c r="M72" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="N72" s="5"/>
+      <c r="N72" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O72" s="5"/>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.25">
@@ -5509,7 +5654,9 @@
       <c r="M73" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="N73" s="5"/>
+      <c r="N73" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O73" s="5"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.25">
@@ -5552,7 +5699,9 @@
       <c r="M74" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="N74" s="5"/>
+      <c r="N74" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O74" s="5"/>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.25">
@@ -5595,7 +5744,9 @@
       <c r="M75" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="N75" s="5"/>
+      <c r="N75" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O75" s="5"/>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.25">
@@ -5638,7 +5789,9 @@
       <c r="M76" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="N76" s="5"/>
+      <c r="N76" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O76" s="5"/>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.25">
@@ -5681,7 +5834,9 @@
       <c r="M77" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="N77" s="5"/>
+      <c r="N77" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O77" s="5"/>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.25">
@@ -5724,7 +5879,9 @@
       <c r="M78" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="N78" s="5"/>
+      <c r="N78" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O78" s="5"/>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.25">
@@ -5767,7 +5924,9 @@
       <c r="M79" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="N79" s="5"/>
+      <c r="N79" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O79" s="5"/>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.25">
@@ -5810,7 +5969,9 @@
       <c r="M80" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="N80" s="5"/>
+      <c r="N80" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O80" s="5"/>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
@@ -5853,7 +6014,9 @@
       <c r="M81" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="N81" s="5"/>
+      <c r="N81" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O81" s="5"/>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
@@ -5896,7 +6059,9 @@
       <c r="M82" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="N82" s="5"/>
+      <c r="N82" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O82" s="5"/>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
@@ -5939,7 +6104,9 @@
       <c r="M83" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="N83" s="5"/>
+      <c r="N83" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O83" s="5"/>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
@@ -5982,7 +6149,9 @@
       <c r="M84" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="N84" s="5"/>
+      <c r="N84" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O84" s="5"/>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.25">
@@ -6025,7 +6194,9 @@
       <c r="M85" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="N85" s="5"/>
+      <c r="N85" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O85" s="5"/>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.25">
@@ -6068,7 +6239,9 @@
       <c r="M86" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="N86" s="5"/>
+      <c r="N86" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O86" s="5"/>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.25">
@@ -6111,7 +6284,9 @@
       <c r="M87" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="N87" s="5"/>
+      <c r="N87" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O87" s="5"/>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.25">
@@ -6154,7 +6329,9 @@
       <c r="M88" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="N88" s="5"/>
+      <c r="N88" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O88" s="5"/>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.25">
@@ -6197,7 +6374,9 @@
       <c r="M89" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="N89" s="5"/>
+      <c r="N89" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O89" s="5"/>
     </row>
     <row r="90" spans="1:15" x14ac:dyDescent="0.25">
@@ -6240,7 +6419,9 @@
       <c r="M90" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N90" s="5"/>
+      <c r="N90" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O90" s="5"/>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.25">
@@ -6283,7 +6464,9 @@
       <c r="M91" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="N91" s="5"/>
+      <c r="N91" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O91" s="5"/>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.25">
@@ -6326,7 +6509,9 @@
       <c r="M92" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="N92" s="5"/>
+      <c r="N92" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O92" s="5"/>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.25">
@@ -6369,7 +6554,9 @@
       <c r="M93" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="N93" s="5"/>
+      <c r="N93" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O93" s="5"/>
     </row>
     <row r="94" spans="1:15" x14ac:dyDescent="0.25">
@@ -6412,7 +6599,9 @@
       <c r="M94" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="N94" s="5"/>
+      <c r="N94" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O94" s="5"/>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.25">
@@ -6455,7 +6644,9 @@
       <c r="M95" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="N95" s="5"/>
+      <c r="N95" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O95" s="5"/>
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.25">
@@ -6498,7 +6689,9 @@
       <c r="M96" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="N96" s="5"/>
+      <c r="N96" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O96" s="5"/>
     </row>
     <row r="97" spans="1:15" x14ac:dyDescent="0.25">
@@ -6541,7 +6734,9 @@
       <c r="M97" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="N97" s="5"/>
+      <c r="N97" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O97" s="5"/>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.25">
@@ -6584,7 +6779,9 @@
       <c r="M98" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="N98" s="5"/>
+      <c r="N98" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O98" s="5"/>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.25">
@@ -6627,7 +6824,9 @@
       <c r="M99" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="N99" s="5"/>
+      <c r="N99" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O99" s="5"/>
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.25">
@@ -6670,7 +6869,9 @@
       <c r="M100" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="N100" s="5"/>
+      <c r="N100" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O100" s="5"/>
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.25">
@@ -6713,7 +6914,9 @@
       <c r="M101" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="N101" s="5"/>
+      <c r="N101" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O101" s="5"/>
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.25">
@@ -6756,7 +6959,9 @@
       <c r="M102" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="N102" s="5"/>
+      <c r="N102" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O102" s="5"/>
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.25">
@@ -6799,7 +7004,9 @@
       <c r="M103" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="N103" s="5"/>
+      <c r="N103" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O103" s="5"/>
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.25">
@@ -6842,7 +7049,9 @@
       <c r="M104" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="N104" s="5"/>
+      <c r="N104" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O104" s="5"/>
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.25">
@@ -6885,7 +7094,9 @@
       <c r="M105" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="N105" s="5"/>
+      <c r="N105" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O105" s="5"/>
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.25">
@@ -6928,7 +7139,9 @@
       <c r="M106" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="N106" s="5"/>
+      <c r="N106" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O106" s="5"/>
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.25">
@@ -6971,7 +7184,9 @@
       <c r="M107" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="N107" s="5"/>
+      <c r="N107" s="5" t="s">
+        <v>643</v>
+      </c>
       <c r="O107" s="5"/>
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: lp register updated
</commit_message>
<xml_diff>
--- a/98 - Excels/Cadastro-LPs.xlsx
+++ b/98 - Excels/Cadastro-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feb3ct\Desktop\PyAutomateSAP\98 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F32C0F4A-DD82-4B8B-8095-3AF23712E3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F29AB4E-E4BF-4ADD-888D-359262AC42BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="140">
   <si>
     <t>Data</t>
   </si>
@@ -437,6 +437,9 @@
   </si>
   <si>
     <t>LP-056145</t>
+  </si>
+  <si>
+    <t>CADASTRADA</t>
   </si>
 </sst>
 </file>
@@ -854,7 +857,8 @@
     <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -944,7 +948,9 @@
       <c r="M2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="N2" s="5"/>
+      <c r="N2" s="5" t="s">
+        <v>139</v>
+      </c>
       <c r="O2" s="5"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -987,7 +993,9 @@
       <c r="M3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="N3" s="5"/>
+      <c r="N3" s="5" t="s">
+        <v>139</v>
+      </c>
       <c r="O3" s="5"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>